<commit_message>
Update parliament data - 2026-03-16
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -113,7 +113,7 @@
     <t xml:space="preserve">&lt;p&gt;Bei der Volksabstimmung vom 8.3.2025 SRG-Initiative hat die SP Schweiz Einnahmen mit angeblichen Rekordkleinstspenden von 1.6 Millionen deklariert. Spenden über 15'000 wurden keine offen gelegt.&amp;nbsp;&lt;br&gt;Kann der Bundesrat bestätigen, dass solche ausserordentlichen Rekordeinnahmen nicht automatisch zu einer Revision führen und dieser Entscheid für eine Revision im Ermessen der EFK liegt?&lt;/p&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">Eingereicht / Déposé</t>
+    <t xml:space="preserve">Erledigt / Liquidé</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267185</t>
@@ -125,6 +125,9 @@
     <t xml:space="preserve">Élu</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-03-16</t>
+  </si>
+  <si>
     <t xml:space="preserve">Staatspolitik</t>
   </si>
   <si>
@@ -201,9 +204,6 @@
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Seit Beginn des Projekts im Jahr 2017 hat die Eidgenössische Finanzkontrolle sechs sehr kritische Prüfberichte zur Steuerung des neuen Auszahlungssystems der Arbeitslosenkassen veröffentlicht.&lt;br&gt;Kann uns der Bundesrat mitteilen, ob das SECO die Bemerkungen der Eidgenössischen Finanzkontrolle ausreichend berücksichtigt hat?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Erledigt / Liquidé</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267129</t>
@@ -11231,17 +11231,19 @@
         <v>36</v>
       </c>
       <c r="R2" t="s">
-        <v>26</v>
-      </c>
-      <c r="S2"/>
+        <v>37</v>
+      </c>
+      <c r="S2" t="s">
+        <v>37</v>
+      </c>
       <c r="T2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="U2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="V2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -11249,63 +11251,65 @@
         <v>20267161</v>
       </c>
       <c r="B3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
         <v>23</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G3" t="s">
         <v>27</v>
       </c>
       <c r="H3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K3"/>
       <c r="L3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N3" t="s">
         <v>33</v>
       </c>
       <c r="O3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="P3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q3" t="s">
         <v>36</v>
       </c>
       <c r="R3" t="s">
-        <v>43</v>
-      </c>
-      <c r="S3"/>
+        <v>37</v>
+      </c>
+      <c r="S3" t="s">
+        <v>37</v>
+      </c>
       <c r="T3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="U3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="V3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4">
@@ -11313,41 +11317,41 @@
         <v>20267129</v>
       </c>
       <c r="B4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C4" t="s">
         <v>23</v>
       </c>
       <c r="D4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G4" t="s">
         <v>27</v>
       </c>
       <c r="H4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K4"/>
       <c r="L4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N4" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O4" t="s">
         <v>64</v>
@@ -11359,7 +11363,7 @@
         <v>36</v>
       </c>
       <c r="R4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="S4"/>
       <c r="T4" t="s">
@@ -11395,7 +11399,7 @@
         <v>27</v>
       </c>
       <c r="H5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I5" t="s">
         <v>74</v>
@@ -11545,7 +11549,7 @@
         <v>111</v>
       </c>
       <c r="N7" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O7" t="s">
         <v>112</v>
@@ -11659,7 +11663,7 @@
         <v>27</v>
       </c>
       <c r="H9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I9" t="s">
         <v>137</v>
@@ -11791,7 +11795,7 @@
         <v>164</v>
       </c>
       <c r="H11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I11" t="s">
         <v>137</v>
@@ -12055,7 +12059,7 @@
         <v>27</v>
       </c>
       <c r="H15" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I15" t="s">
         <v>209</v>
@@ -12121,7 +12125,7 @@
         <v>164</v>
       </c>
       <c r="H16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I16" t="s">
         <v>222</v>
@@ -12139,7 +12143,7 @@
         <v>226</v>
       </c>
       <c r="N16" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O16" t="s">
         <v>227</v>
@@ -12269,7 +12273,7 @@
         <v>250</v>
       </c>
       <c r="N18" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O18" t="s">
         <v>251</v>
@@ -12335,7 +12339,7 @@
         <v>262</v>
       </c>
       <c r="N19" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O19" t="s">
         <v>263</v>
@@ -12383,7 +12387,7 @@
         <v>27</v>
       </c>
       <c r="H20" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I20" t="s">
         <v>272</v>
@@ -12449,7 +12453,7 @@
         <v>27</v>
       </c>
       <c r="H21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I21" t="s">
         <v>285</v>
@@ -12581,7 +12585,7 @@
         <v>27</v>
       </c>
       <c r="H23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I23" t="s">
         <v>311</v>
@@ -12797,7 +12801,7 @@
         <v>353</v>
       </c>
       <c r="N26" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O26" t="s">
         <v>354</v>
@@ -12863,7 +12867,7 @@
         <v>366</v>
       </c>
       <c r="N27" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O27" t="s">
         <v>367</v>
@@ -12929,7 +12933,7 @@
         <v>378</v>
       </c>
       <c r="N28" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O28" t="s">
         <v>379</v>
@@ -12995,7 +12999,7 @@
         <v>390</v>
       </c>
       <c r="N29" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O29" t="s">
         <v>391</v>
@@ -13061,7 +13065,7 @@
         <v>401</v>
       </c>
       <c r="N30" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O30" t="s">
         <v>402</v>
@@ -13109,7 +13113,7 @@
         <v>27</v>
       </c>
       <c r="H31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I31" t="s">
         <v>407</v>
@@ -13175,7 +13179,7 @@
         <v>27</v>
       </c>
       <c r="H32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I32" t="s">
         <v>419</v>
@@ -13191,7 +13195,7 @@
         <v>422</v>
       </c>
       <c r="N32" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O32" t="s">
         <v>423</v>
@@ -13321,7 +13325,7 @@
         <v>446</v>
       </c>
       <c r="N34" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O34" t="s">
         <v>447</v>
@@ -13385,7 +13389,7 @@
         <v>456</v>
       </c>
       <c r="N35" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O35" t="s">
         <v>457</v>
@@ -13449,7 +13453,7 @@
         <v>467</v>
       </c>
       <c r="N36" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O36" t="s">
         <v>468</v>
@@ -13579,7 +13583,7 @@
         <v>490</v>
       </c>
       <c r="N38" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O38" t="s">
         <v>491</v>
@@ -13643,7 +13647,7 @@
         <v>503</v>
       </c>
       <c r="N39" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O39" t="s">
         <v>504</v>
@@ -13709,7 +13713,7 @@
         <v>513</v>
       </c>
       <c r="N40" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O40" t="s">
         <v>514</v>
@@ -13775,7 +13779,7 @@
         <v>524</v>
       </c>
       <c r="N41" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O41" t="s">
         <v>525</v>
@@ -13823,7 +13827,7 @@
         <v>27</v>
       </c>
       <c r="H42" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I42" t="s">
         <v>533</v>
@@ -13839,7 +13843,7 @@
         <v>536</v>
       </c>
       <c r="N42" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O42" t="s">
         <v>537</v>
@@ -14151,7 +14155,7 @@
         <v>27</v>
       </c>
       <c r="H47" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I47" t="s">
         <v>591</v>
@@ -14217,7 +14221,7 @@
         <v>27</v>
       </c>
       <c r="H48" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I48" t="s">
         <v>599</v>
@@ -14283,7 +14287,7 @@
         <v>27</v>
       </c>
       <c r="H49" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I49" t="s">
         <v>610</v>
@@ -14349,7 +14353,7 @@
         <v>27</v>
       </c>
       <c r="H50" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I50" t="s">
         <v>619</v>
@@ -14433,7 +14437,7 @@
         <v>636</v>
       </c>
       <c r="N51" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O51" t="s">
         <v>637</v>
@@ -14497,7 +14501,7 @@
         <v>644</v>
       </c>
       <c r="N52" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O52" t="s">
         <v>645</v>
@@ -14545,7 +14549,7 @@
         <v>27</v>
       </c>
       <c r="H53" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I53" t="s">
         <v>651</v>
@@ -14561,7 +14565,7 @@
         <v>654</v>
       </c>
       <c r="N53" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O53" t="s">
         <v>655</v>
@@ -14609,7 +14613,7 @@
         <v>27</v>
       </c>
       <c r="H54" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I54" t="s">
         <v>663</v>
@@ -14625,7 +14629,7 @@
         <v>666</v>
       </c>
       <c r="N54" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O54" t="s">
         <v>667</v>
@@ -14673,7 +14677,7 @@
         <v>27</v>
       </c>
       <c r="H55" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I55" t="s">
         <v>673</v>
@@ -14689,7 +14693,7 @@
         <v>676</v>
       </c>
       <c r="N55" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O55" t="s">
         <v>677</v>
@@ -14819,7 +14823,7 @@
         <v>697</v>
       </c>
       <c r="N57" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O57" t="s">
         <v>698</v>
@@ -14867,7 +14871,7 @@
         <v>27</v>
       </c>
       <c r="H58" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I58" t="s">
         <v>702</v>
@@ -14883,7 +14887,7 @@
         <v>705</v>
       </c>
       <c r="N58" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O58" t="s">
         <v>706</v>
@@ -14997,7 +15001,7 @@
         <v>27</v>
       </c>
       <c r="H60" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I60" t="s">
         <v>724</v>
@@ -15081,7 +15085,7 @@
         <v>739</v>
       </c>
       <c r="N61" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O61" t="s">
         <v>740</v>
@@ -15147,7 +15151,7 @@
         <v>751</v>
       </c>
       <c r="N62" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O62" t="s">
         <v>752</v>
@@ -15213,7 +15217,7 @@
         <v>761</v>
       </c>
       <c r="N63" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O63" t="s">
         <v>762</v>
@@ -15277,7 +15281,7 @@
         <v>771</v>
       </c>
       <c r="N64" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O64" t="s">
         <v>772</v>
@@ -15323,7 +15327,7 @@
         <v>27</v>
       </c>
       <c r="H65" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I65" t="s">
         <v>777</v>
@@ -15473,7 +15477,7 @@
         <v>804</v>
       </c>
       <c r="N67" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O67" t="s">
         <v>805</v>
@@ -15539,7 +15543,7 @@
         <v>813</v>
       </c>
       <c r="N68" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O68" t="s">
         <v>814</v>
@@ -15605,7 +15609,7 @@
         <v>826</v>
       </c>
       <c r="N69" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O69" t="s">
         <v>827</v>
@@ -15653,7 +15657,7 @@
         <v>27</v>
       </c>
       <c r="H70" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I70" t="s">
         <v>832</v>
@@ -15669,7 +15673,7 @@
         <v>835</v>
       </c>
       <c r="N70" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O70" t="s">
         <v>836</v>
@@ -15733,7 +15737,7 @@
         <v>846</v>
       </c>
       <c r="N71" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O71" t="s">
         <v>847</v>
@@ -15781,7 +15785,7 @@
         <v>27</v>
       </c>
       <c r="H72" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I72" t="s">
         <v>851</v>
@@ -15799,7 +15803,7 @@
         <v>855</v>
       </c>
       <c r="N72" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O72" t="s">
         <v>856</v>
@@ -15865,7 +15869,7 @@
         <v>868</v>
       </c>
       <c r="N73" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O73" t="s">
         <v>869</v>
@@ -15913,7 +15917,7 @@
         <v>27</v>
       </c>
       <c r="H74" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I74" t="s">
         <v>877</v>
@@ -15931,7 +15935,7 @@
         <v>881</v>
       </c>
       <c r="N74" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O74" t="s">
         <v>882</v>
@@ -15997,7 +16001,7 @@
         <v>894</v>
       </c>
       <c r="N75" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O75" t="s">
         <v>895</v>
@@ -16061,7 +16065,7 @@
         <v>907</v>
       </c>
       <c r="N76" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O76" t="s">
         <v>908</v>
@@ -16127,7 +16131,7 @@
         <v>920</v>
       </c>
       <c r="N77" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O77" t="s">
         <v>921</v>
@@ -16169,7 +16173,7 @@
         <v>27</v>
       </c>
       <c r="H78" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I78" t="s">
         <v>925</v>
@@ -16185,7 +16189,7 @@
         <v>928</v>
       </c>
       <c r="N78" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O78" t="s">
         <v>929</v>
@@ -16251,7 +16255,7 @@
         <v>940</v>
       </c>
       <c r="N79" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O79" t="s">
         <v>941</v>
@@ -16299,7 +16303,7 @@
         <v>27</v>
       </c>
       <c r="H80" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I80" t="s">
         <v>944</v>
@@ -16317,7 +16321,7 @@
         <v>948</v>
       </c>
       <c r="N80" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O80" t="s">
         <v>949</v>
@@ -16383,7 +16387,7 @@
         <v>958</v>
       </c>
       <c r="N81" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O81" t="s">
         <v>959</v>
@@ -16515,7 +16519,7 @@
         <v>983</v>
       </c>
       <c r="N83" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O83" t="s">
         <v>984</v>
@@ -16581,7 +16585,7 @@
         <v>995</v>
       </c>
       <c r="N84" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O84" t="s">
         <v>996</v>
@@ -16647,7 +16651,7 @@
         <v>1004</v>
       </c>
       <c r="N85" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O85" t="s">
         <v>1005</v>
@@ -16695,7 +16699,7 @@
         <v>27</v>
       </c>
       <c r="H86" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I86" t="s">
         <v>1011</v>
@@ -16713,7 +16717,7 @@
         <v>1015</v>
       </c>
       <c r="N86" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O86" t="s">
         <v>1016</v>
@@ -16779,7 +16783,7 @@
         <v>1027</v>
       </c>
       <c r="N87" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O87" t="s">
         <v>1028</v>
@@ -16827,7 +16831,7 @@
         <v>27</v>
       </c>
       <c r="H88" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I88" t="s">
         <v>1036</v>
@@ -16845,7 +16849,7 @@
         <v>1040</v>
       </c>
       <c r="N88" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O88" t="s">
         <v>1041</v>
@@ -16893,7 +16897,7 @@
         <v>27</v>
       </c>
       <c r="H89" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I89" t="s">
         <v>1049</v>
@@ -16911,7 +16915,7 @@
         <v>1053</v>
       </c>
       <c r="N89" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O89" t="s">
         <v>1054</v>
@@ -16977,7 +16981,7 @@
         <v>1065</v>
       </c>
       <c r="N90" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O90" t="s">
         <v>1066</v>
@@ -17025,7 +17029,7 @@
         <v>27</v>
       </c>
       <c r="H91" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I91" t="s">
         <v>1072</v>
@@ -17043,7 +17047,7 @@
         <v>1076</v>
       </c>
       <c r="N91" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O91" t="s">
         <v>1077</v>
@@ -17091,7 +17095,7 @@
         <v>27</v>
       </c>
       <c r="H92" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I92" t="s">
         <v>1081</v>
@@ -17109,7 +17113,7 @@
         <v>1085</v>
       </c>
       <c r="N92" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O92" t="s">
         <v>1086</v>
@@ -17175,7 +17179,7 @@
         <v>1095</v>
       </c>
       <c r="N93" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O93" t="s">
         <v>1096</v>
@@ -17211,7 +17215,7 @@
         <v>135</v>
       </c>
       <c r="D94" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E94" t="s">
         <v>270</v>
@@ -17241,7 +17245,7 @@
         <v>1107</v>
       </c>
       <c r="N94" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O94" t="s">
         <v>1108</v>
@@ -17277,7 +17281,7 @@
         <v>135</v>
       </c>
       <c r="D95" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E95" t="s">
         <v>270</v>
@@ -17307,7 +17311,7 @@
         <v>1118</v>
       </c>
       <c r="N95" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O95" t="s">
         <v>1119</v>
@@ -17355,7 +17359,7 @@
         <v>27</v>
       </c>
       <c r="H96" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I96" t="s">
         <v>1127</v>
@@ -17373,7 +17377,7 @@
         <v>1131</v>
       </c>
       <c r="N96" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O96" t="s">
         <v>1132</v>
@@ -17421,7 +17425,7 @@
         <v>27</v>
       </c>
       <c r="H97" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I97" t="s">
         <v>1138</v>
@@ -17439,7 +17443,7 @@
         <v>1142</v>
       </c>
       <c r="N97" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O97" t="s">
         <v>1143</v>
@@ -17505,7 +17509,7 @@
         <v>1153</v>
       </c>
       <c r="N98" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O98" t="s">
         <v>1154</v>
@@ -17553,7 +17557,7 @@
         <v>27</v>
       </c>
       <c r="H99" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I99" t="s">
         <v>1159</v>
@@ -17571,7 +17575,7 @@
         <v>1163</v>
       </c>
       <c r="N99" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O99" t="s">
         <v>1164</v>
@@ -17637,7 +17641,7 @@
         <v>1174</v>
       </c>
       <c r="N100" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O100" t="s">
         <v>1175</v>
@@ -17703,7 +17707,7 @@
         <v>1185</v>
       </c>
       <c r="N101" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O101" t="s">
         <v>1186</v>
@@ -17769,7 +17773,7 @@
         <v>1194</v>
       </c>
       <c r="N102" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O102" t="s">
         <v>1195</v>
@@ -17899,7 +17903,7 @@
         <v>1211</v>
       </c>
       <c r="N104" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O104" t="s">
         <v>1212</v>
@@ -17963,7 +17967,7 @@
         <v>1221</v>
       </c>
       <c r="N105" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O105" t="s">
         <v>1222</v>
@@ -18029,7 +18033,7 @@
         <v>1234</v>
       </c>
       <c r="N106" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O106" t="s">
         <v>1235</v>
@@ -18077,7 +18081,7 @@
         <v>27</v>
       </c>
       <c r="H107" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I107" t="s">
         <v>1241</v>
@@ -18095,7 +18099,7 @@
         <v>1245</v>
       </c>
       <c r="N107" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O107" t="s">
         <v>1246</v>
@@ -18161,7 +18165,7 @@
         <v>1255</v>
       </c>
       <c r="N108" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O108" t="s">
         <v>1256</v>
@@ -18209,7 +18213,7 @@
         <v>27</v>
       </c>
       <c r="H109" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I109" t="s">
         <v>1260</v>
@@ -18227,7 +18231,7 @@
         <v>1264</v>
       </c>
       <c r="N109" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O109" t="s">
         <v>1265</v>
@@ -18275,7 +18279,7 @@
         <v>27</v>
       </c>
       <c r="H110" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I110" t="s">
         <v>1273</v>
@@ -18357,7 +18361,7 @@
         <v>1289</v>
       </c>
       <c r="N111" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O111" t="s">
         <v>1290</v>
@@ -18421,7 +18425,7 @@
         <v>1298</v>
       </c>
       <c r="N112" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O112" t="s">
         <v>1299</v>
@@ -18485,7 +18489,7 @@
         <v>1310</v>
       </c>
       <c r="N113" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O113" t="s">
         <v>1311</v>
@@ -18533,7 +18537,7 @@
         <v>27</v>
       </c>
       <c r="H114" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I114" t="s">
         <v>1316</v>
@@ -18551,7 +18555,7 @@
         <v>1320</v>
       </c>
       <c r="N114" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O114" t="s">
         <v>1321</v>
@@ -18617,7 +18621,7 @@
         <v>1332</v>
       </c>
       <c r="N115" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O115" t="s">
         <v>1333</v>
@@ -18681,7 +18685,7 @@
         <v>1345</v>
       </c>
       <c r="N116" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O116" t="s">
         <v>1346</v>
@@ -18729,7 +18733,7 @@
         <v>27</v>
       </c>
       <c r="H117" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I117" t="s">
         <v>1353</v>
@@ -18745,7 +18749,7 @@
         <v>1356</v>
       </c>
       <c r="N117" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O117" t="s">
         <v>1357</v>
@@ -18811,7 +18815,7 @@
         <v>1369</v>
       </c>
       <c r="N118" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O118" t="s">
         <v>1370</v>
@@ -18877,7 +18881,7 @@
         <v>1382</v>
       </c>
       <c r="N119" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O119" t="s">
         <v>1383</v>
@@ -18925,7 +18929,7 @@
         <v>27</v>
       </c>
       <c r="H120" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I120" t="s">
         <v>1391</v>
@@ -18941,7 +18945,7 @@
         <v>1394</v>
       </c>
       <c r="N120" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O120" t="s">
         <v>1395</v>
@@ -19007,7 +19011,7 @@
         <v>1407</v>
       </c>
       <c r="N121" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O121" t="s">
         <v>1408</v>
@@ -19073,7 +19077,7 @@
         <v>1420</v>
       </c>
       <c r="N122" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O122" t="s">
         <v>1421</v>
@@ -19139,7 +19143,7 @@
         <v>1431</v>
       </c>
       <c r="N123" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O123" t="s">
         <v>1432</v>
@@ -19205,7 +19209,7 @@
         <v>1440</v>
       </c>
       <c r="N124" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O124" t="s">
         <v>1441</v>
@@ -19271,7 +19275,7 @@
         <v>1453</v>
       </c>
       <c r="N125" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O125" t="s">
         <v>1454</v>
@@ -19319,7 +19323,7 @@
         <v>27</v>
       </c>
       <c r="H126" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I126" t="s">
         <v>1461</v>
@@ -19335,7 +19339,7 @@
         <v>1464</v>
       </c>
       <c r="N126" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O126" t="s">
         <v>1465</v>
@@ -19383,7 +19387,7 @@
         <v>27</v>
       </c>
       <c r="H127" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I127" t="s">
         <v>1473</v>
@@ -19399,7 +19403,7 @@
         <v>1476</v>
       </c>
       <c r="N127" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O127" t="s">
         <v>1477</v>
@@ -19529,7 +19533,7 @@
         <v>1495</v>
       </c>
       <c r="N129" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O129" t="s">
         <v>1496</v>
@@ -19577,7 +19581,7 @@
         <v>27</v>
       </c>
       <c r="H130" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I130" t="s">
         <v>1503</v>
@@ -19595,7 +19599,7 @@
         <v>1507</v>
       </c>
       <c r="N130" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O130" t="s">
         <v>1508</v>
@@ -19643,7 +19647,7 @@
         <v>27</v>
       </c>
       <c r="H131" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I131" t="s">
         <v>1514</v>
@@ -19661,7 +19665,7 @@
         <v>1518</v>
       </c>
       <c r="N131" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O131" t="s">
         <v>1519</v>
@@ -19727,7 +19731,7 @@
         <v>1530</v>
       </c>
       <c r="N132" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O132" t="s">
         <v>1531</v>
@@ -19775,7 +19779,7 @@
         <v>164</v>
       </c>
       <c r="H133" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I133" t="s">
         <v>1539</v>
@@ -19841,7 +19845,7 @@
         <v>27</v>
       </c>
       <c r="H134" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I134" t="s">
         <v>1551</v>
@@ -19859,7 +19863,7 @@
         <v>1555</v>
       </c>
       <c r="N134" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O134" t="s">
         <v>1556</v>
@@ -19925,7 +19929,7 @@
         <v>1567</v>
       </c>
       <c r="N135" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O135" t="s">
         <v>1568</v>
@@ -19991,7 +19995,7 @@
         <v>1576</v>
       </c>
       <c r="N136" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O136" t="s">
         <v>1577</v>
@@ -20055,7 +20059,7 @@
         <v>1585</v>
       </c>
       <c r="N137" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O137" t="s">
         <v>1586</v>
@@ -20119,7 +20123,7 @@
         <v>1592</v>
       </c>
       <c r="N138" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O138" t="s">
         <v>1593</v>
@@ -20185,7 +20189,7 @@
         <v>1601</v>
       </c>
       <c r="N139" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O139" t="s">
         <v>1602</v>
@@ -20251,7 +20255,7 @@
         <v>1613</v>
       </c>
       <c r="N140" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O140" t="s">
         <v>1614</v>
@@ -20317,7 +20321,7 @@
         <v>1624</v>
       </c>
       <c r="N141" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O141" t="s">
         <v>1625</v>
@@ -20383,7 +20387,7 @@
         <v>1636</v>
       </c>
       <c r="N142" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O142" t="s">
         <v>1637</v>
@@ -20449,7 +20453,7 @@
         <v>1645</v>
       </c>
       <c r="N143" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O143" t="s">
         <v>1646</v>
@@ -20515,7 +20519,7 @@
         <v>1657</v>
       </c>
       <c r="N144" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O144" t="s">
         <v>1658</v>
@@ -20581,7 +20585,7 @@
         <v>1669</v>
       </c>
       <c r="N145" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O145" t="s">
         <v>1670</v>
@@ -20647,7 +20651,7 @@
         <v>1678</v>
       </c>
       <c r="N146" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O146" t="s">
         <v>1679</v>
@@ -20711,7 +20715,7 @@
         <v>1690</v>
       </c>
       <c r="N147" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O147" t="s">
         <v>1691</v>
@@ -20775,7 +20779,7 @@
         <v>1701</v>
       </c>
       <c r="N148" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O148" t="s">
         <v>1702</v>
@@ -20839,7 +20843,7 @@
         <v>1708</v>
       </c>
       <c r="N149" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O149" t="s">
         <v>1709</v>
@@ -20949,7 +20953,7 @@
         <v>27</v>
       </c>
       <c r="H151" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I151" t="s">
         <v>1724</v>
@@ -20967,7 +20971,7 @@
         <v>1728</v>
       </c>
       <c r="N151" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O151" t="s">
         <v>1729</v>
@@ -21033,7 +21037,7 @@
         <v>1740</v>
       </c>
       <c r="N152" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O152" t="s">
         <v>1741</v>
@@ -21099,7 +21103,7 @@
         <v>1752</v>
       </c>
       <c r="N153" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O153" t="s">
         <v>1753</v>
@@ -21165,7 +21169,7 @@
         <v>1765</v>
       </c>
       <c r="N154" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O154" t="s">
         <v>1766</v>
@@ -21229,7 +21233,7 @@
         <v>1774</v>
       </c>
       <c r="N155" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O155" t="s">
         <v>1775</v>
@@ -21295,7 +21299,7 @@
         <v>1787</v>
       </c>
       <c r="N156" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O156" t="s">
         <v>1788</v>
@@ -21361,7 +21365,7 @@
         <v>1799</v>
       </c>
       <c r="N157" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O157" t="s">
         <v>1800</v>
@@ -21427,7 +21431,7 @@
         <v>1811</v>
       </c>
       <c r="N158" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O158" t="s">
         <v>1812</v>
@@ -21493,7 +21497,7 @@
         <v>1823</v>
       </c>
       <c r="N159" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O159" t="s">
         <v>1824</v>
@@ -21541,7 +21545,7 @@
         <v>27</v>
       </c>
       <c r="H160" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I160" t="s">
         <v>1830</v>
@@ -21559,7 +21563,7 @@
         <v>1834</v>
       </c>
       <c r="N160" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O160" t="s">
         <v>1835</v>
@@ -21607,7 +21611,7 @@
         <v>27</v>
       </c>
       <c r="H161" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I161" t="s">
         <v>1841</v>
@@ -21625,7 +21629,7 @@
         <v>1845</v>
       </c>
       <c r="N161" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O161" t="s">
         <v>1846</v>
@@ -21691,7 +21695,7 @@
         <v>1854</v>
       </c>
       <c r="N162" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O162" t="s">
         <v>1855</v>
@@ -21757,7 +21761,7 @@
         <v>1864</v>
       </c>
       <c r="N163" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O163" t="s">
         <v>1865</v>
@@ -21805,7 +21809,7 @@
         <v>27</v>
       </c>
       <c r="H164" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I164" t="s">
         <v>1872</v>
@@ -21823,7 +21827,7 @@
         <v>1876</v>
       </c>
       <c r="N164" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O164" t="s">
         <v>1877</v>
@@ -21889,7 +21893,7 @@
         <v>1888</v>
       </c>
       <c r="N165" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O165" t="s">
         <v>1889</v>
@@ -21955,7 +21959,7 @@
         <v>1897</v>
       </c>
       <c r="N166" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O166" t="s">
         <v>1898</v>
@@ -22021,7 +22025,7 @@
         <v>1906</v>
       </c>
       <c r="N167" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O167" t="s">
         <v>1907</v>
@@ -22087,7 +22091,7 @@
         <v>1919</v>
       </c>
       <c r="N168" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O168" t="s">
         <v>1920</v>
@@ -22153,7 +22157,7 @@
         <v>1931</v>
       </c>
       <c r="N169" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O169" t="s">
         <v>1932</v>
@@ -22201,7 +22205,7 @@
         <v>27</v>
       </c>
       <c r="H170" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I170" t="s">
         <v>1939</v>
@@ -22219,7 +22223,7 @@
         <v>1943</v>
       </c>
       <c r="N170" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O170" t="s">
         <v>1944</v>
@@ -22267,7 +22271,7 @@
         <v>27</v>
       </c>
       <c r="H171" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I171" t="s">
         <v>1951</v>
@@ -22285,7 +22289,7 @@
         <v>1955</v>
       </c>
       <c r="N171" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O171" t="s">
         <v>1956</v>
@@ -22351,7 +22355,7 @@
         <v>1967</v>
       </c>
       <c r="N172" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O172" t="s">
         <v>1968</v>
@@ -22399,7 +22403,7 @@
         <v>27</v>
       </c>
       <c r="H173" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I173" t="s">
         <v>1973</v>
@@ -22417,7 +22421,7 @@
         <v>1977</v>
       </c>
       <c r="N173" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O173" t="s">
         <v>1978</v>
@@ -22481,7 +22485,7 @@
         <v>1985</v>
       </c>
       <c r="N174" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O174" t="s">
         <v>1986</v>
@@ -22545,7 +22549,7 @@
         <v>1996</v>
       </c>
       <c r="N175" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O175" t="s">
         <v>1997</v>
@@ -22611,7 +22615,7 @@
         <v>2008</v>
       </c>
       <c r="N176" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O176" t="s">
         <v>2009</v>
@@ -22659,7 +22663,7 @@
         <v>27</v>
       </c>
       <c r="H177" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I177" t="s">
         <v>2016</v>
@@ -22677,7 +22681,7 @@
         <v>2020</v>
       </c>
       <c r="N177" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O177" t="s">
         <v>2021</v>
@@ -22725,7 +22729,7 @@
         <v>27</v>
       </c>
       <c r="H178" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I178" t="s">
         <v>2030</v>
@@ -22743,7 +22747,7 @@
         <v>2034</v>
       </c>
       <c r="N178" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O178" t="s">
         <v>2035</v>
@@ -22809,7 +22813,7 @@
         <v>2045</v>
       </c>
       <c r="N179" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O179" t="s">
         <v>2046</v>
@@ -22875,7 +22879,7 @@
         <v>2058</v>
       </c>
       <c r="N180" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O180" t="s">
         <v>2059</v>
@@ -22923,7 +22927,7 @@
         <v>27</v>
       </c>
       <c r="H181" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I181" t="s">
         <v>2067</v>
@@ -22939,7 +22943,7 @@
         <v>2070</v>
       </c>
       <c r="N181" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O181" t="s">
         <v>2071</v>
@@ -22987,7 +22991,7 @@
         <v>27</v>
       </c>
       <c r="H182" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I182" t="s">
         <v>2078</v>
@@ -23005,7 +23009,7 @@
         <v>2082</v>
       </c>
       <c r="N182" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O182" t="s">
         <v>2083</v>
@@ -23071,7 +23075,7 @@
         <v>2094</v>
       </c>
       <c r="N183" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O183" t="s">
         <v>2095</v>
@@ -23135,7 +23139,7 @@
         <v>2103</v>
       </c>
       <c r="N184" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O184" t="s">
         <v>2104</v>
@@ -23183,7 +23187,7 @@
         <v>27</v>
       </c>
       <c r="H185" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I185" t="s">
         <v>2112</v>
@@ -23201,7 +23205,7 @@
         <v>2116</v>
       </c>
       <c r="N185" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O185" t="s">
         <v>2117</v>
@@ -23249,7 +23253,7 @@
         <v>27</v>
       </c>
       <c r="H186" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I186" t="s">
         <v>2125</v>
@@ -23267,7 +23271,7 @@
         <v>2129</v>
       </c>
       <c r="N186" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O186" t="s">
         <v>2130</v>
@@ -23315,7 +23319,7 @@
         <v>27</v>
       </c>
       <c r="H187" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I187" t="s">
         <v>2137</v>
@@ -23331,7 +23335,7 @@
         <v>2140</v>
       </c>
       <c r="N187" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O187" t="s">
         <v>2141</v>
@@ -23379,7 +23383,7 @@
         <v>27</v>
       </c>
       <c r="H188" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I188" t="s">
         <v>2148</v>
@@ -23397,7 +23401,7 @@
         <v>2152</v>
       </c>
       <c r="N188" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O188" t="s">
         <v>2153</v>
@@ -23461,7 +23465,7 @@
         <v>2165</v>
       </c>
       <c r="N189" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O189" t="s">
         <v>2166</v>
@@ -23525,7 +23529,7 @@
         <v>2178</v>
       </c>
       <c r="N190" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O190" t="s">
         <v>2179</v>
@@ -23571,7 +23575,7 @@
         <v>164</v>
       </c>
       <c r="H191" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I191" t="s">
         <v>2185</v>
@@ -23589,7 +23593,7 @@
         <v>2189</v>
       </c>
       <c r="N191" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O191" t="s">
         <v>2190</v>
@@ -23829,7 +23833,7 @@
         <v>27</v>
       </c>
       <c r="H195" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I195" t="s">
         <v>2230</v>
@@ -23884,7 +23888,7 @@
         <v>373</v>
       </c>
       <c r="E196" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F196" t="s">
         <v>89</v>
@@ -23893,7 +23897,7 @@
         <v>27</v>
       </c>
       <c r="H196" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I196" t="s">
         <v>2241</v>
@@ -23948,7 +23952,7 @@
         <v>2252</v>
       </c>
       <c r="E197" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F197" t="s">
         <v>89</v>
@@ -24012,7 +24016,7 @@
         <v>808</v>
       </c>
       <c r="E198" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F198" t="s">
         <v>89</v>
@@ -24101,7 +24105,7 @@
         <v>2278</v>
       </c>
       <c r="N199" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O199" t="s">
         <v>2279</v>
@@ -24163,7 +24167,7 @@
         <v>2285</v>
       </c>
       <c r="N200" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O200" t="s">
         <v>2286</v>
@@ -24227,7 +24231,7 @@
         <v>2297</v>
       </c>
       <c r="N201" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O201" t="s">
         <v>2298</v>
@@ -24264,7 +24268,7 @@
         <v>2301</v>
       </c>
       <c r="E202" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F202" t="s">
         <v>2302</v>
@@ -24273,7 +24277,7 @@
         <v>27</v>
       </c>
       <c r="H202" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I202" t="s">
         <v>2303</v>
@@ -24337,7 +24341,7 @@
         <v>27</v>
       </c>
       <c r="H203" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I203" t="s">
         <v>2311</v>
@@ -24419,7 +24423,7 @@
         <v>2328</v>
       </c>
       <c r="N204" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O204" t="s">
         <v>2329</v>
@@ -24584,7 +24588,7 @@
         <v>2352</v>
       </c>
       <c r="E207" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F207" t="s">
         <v>2323</v>
@@ -24611,7 +24615,7 @@
         <v>2357</v>
       </c>
       <c r="N207" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O207" t="s">
         <v>2358</v>
@@ -24675,7 +24679,7 @@
         <v>2370</v>
       </c>
       <c r="N208" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O208" t="s">
         <v>2371</v>
@@ -24712,7 +24716,7 @@
         <v>442</v>
       </c>
       <c r="E209" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F209" t="s">
         <v>2377</v>
@@ -24801,7 +24805,7 @@
         <v>2389</v>
       </c>
       <c r="N210" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O210" t="s">
         <v>2390</v>
@@ -24863,7 +24867,7 @@
         <v>2396</v>
       </c>
       <c r="N211" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O211" t="s">
         <v>2397</v>
@@ -24909,7 +24913,7 @@
         <v>27</v>
       </c>
       <c r="H212" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I212" t="s">
         <v>2403</v>
@@ -24925,7 +24929,7 @@
         <v>2406</v>
       </c>
       <c r="N212" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O212" t="s">
         <v>2407</v>
@@ -25111,7 +25115,7 @@
         <v>2433</v>
       </c>
       <c r="N215" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O215" t="s">
         <v>2434</v>
@@ -25148,7 +25152,7 @@
         <v>2440</v>
       </c>
       <c r="E216" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F216" t="s">
         <v>2424</v>
@@ -25173,7 +25177,7 @@
         <v>2444</v>
       </c>
       <c r="N216" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O216" t="s">
         <v>2445</v>
@@ -25219,7 +25223,7 @@
         <v>164</v>
       </c>
       <c r="H217" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I217" t="s">
         <v>2450</v>
@@ -25237,7 +25241,7 @@
         <v>2454</v>
       </c>
       <c r="N217" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O217" t="s">
         <v>2455</v>
@@ -25299,7 +25303,7 @@
         <v>2462</v>
       </c>
       <c r="N218" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O218" t="s">
         <v>2463</v>
@@ -25419,7 +25423,7 @@
         <v>2482</v>
       </c>
       <c r="N220" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O220" t="s">
         <v>2483</v>
@@ -25483,7 +25487,7 @@
         <v>2494</v>
       </c>
       <c r="N221" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O221" t="s">
         <v>2495</v>
@@ -25529,7 +25533,7 @@
         <v>27</v>
       </c>
       <c r="H222" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I222" t="s">
         <v>2503</v>
@@ -25547,7 +25551,7 @@
         <v>2507</v>
       </c>
       <c r="N222" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O222" t="s">
         <v>2508</v>
@@ -25609,7 +25613,7 @@
         <v>2518</v>
       </c>
       <c r="N223" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O223" t="s">
         <v>2519</v>
@@ -25655,7 +25659,7 @@
         <v>27</v>
       </c>
       <c r="H224" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I224" t="s">
         <v>2524</v>
@@ -25673,7 +25677,7 @@
         <v>2528</v>
       </c>
       <c r="N224" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O224" t="s">
         <v>2529</v>
@@ -25737,7 +25741,7 @@
         <v>2539</v>
       </c>
       <c r="N225" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O225" t="s">
         <v>2540</v>
@@ -25801,7 +25805,7 @@
         <v>2548</v>
       </c>
       <c r="N226" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O226" t="s">
         <v>2549</v>
@@ -25865,7 +25869,7 @@
         <v>2560</v>
       </c>
       <c r="N227" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O227" t="s">
         <v>2561</v>
@@ -25929,7 +25933,7 @@
         <v>2569</v>
       </c>
       <c r="N228" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O228" t="s">
         <v>2570</v>
@@ -25975,7 +25979,7 @@
         <v>27</v>
       </c>
       <c r="H229" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I229" t="s">
         <v>2574</v>
@@ -25993,7 +25997,7 @@
         <v>2578</v>
       </c>
       <c r="N229" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O229" t="s">
         <v>2579</v>
@@ -26057,7 +26061,7 @@
         <v>2590</v>
       </c>
       <c r="N230" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O230" t="s">
         <v>2591</v>
@@ -26103,7 +26107,7 @@
         <v>27</v>
       </c>
       <c r="H231" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I231" t="s">
         <v>2595</v>
@@ -26121,7 +26125,7 @@
         <v>2599</v>
       </c>
       <c r="N231" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O231" t="s">
         <v>2600</v>
@@ -26185,7 +26189,7 @@
         <v>2612</v>
       </c>
       <c r="N232" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O232" t="s">
         <v>2613</v>
@@ -26247,7 +26251,7 @@
         <v>2623</v>
       </c>
       <c r="N233" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O233" t="s">
         <v>2624</v>
@@ -26311,7 +26315,7 @@
         <v>2635</v>
       </c>
       <c r="N234" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O234" t="s">
         <v>2636</v>
@@ -26375,7 +26379,7 @@
         <v>2648</v>
       </c>
       <c r="N235" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O235" t="s">
         <v>2649</v>
@@ -26439,7 +26443,7 @@
         <v>2659</v>
       </c>
       <c r="N236" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O236" t="s">
         <v>2660</v>
@@ -26485,7 +26489,7 @@
         <v>27</v>
       </c>
       <c r="H237" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I237" t="s">
         <v>2666</v>
@@ -26503,7 +26507,7 @@
         <v>2670</v>
       </c>
       <c r="N237" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O237" t="s">
         <v>2671</v>
@@ -26567,7 +26571,7 @@
         <v>2682</v>
       </c>
       <c r="N238" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O238" t="s">
         <v>2683</v>
@@ -26631,7 +26635,7 @@
         <v>2694</v>
       </c>
       <c r="N239" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O239" t="s">
         <v>2695</v>
@@ -26695,7 +26699,7 @@
         <v>2707</v>
       </c>
       <c r="N240" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O240" t="s">
         <v>2708</v>
@@ -26759,7 +26763,7 @@
         <v>2721</v>
       </c>
       <c r="N241" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O241" t="s">
         <v>2722</v>
@@ -26805,7 +26809,7 @@
         <v>27</v>
       </c>
       <c r="H242" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I242" t="s">
         <v>2727</v>
@@ -26821,7 +26825,7 @@
         <v>2730</v>
       </c>
       <c r="N242" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O242" t="s">
         <v>2731</v>
@@ -26867,7 +26871,7 @@
         <v>27</v>
       </c>
       <c r="H243" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I243" t="s">
         <v>2734</v>
@@ -26883,7 +26887,7 @@
         <v>2737</v>
       </c>
       <c r="N243" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O243" t="s">
         <v>2738</v>
@@ -26929,7 +26933,7 @@
         <v>27</v>
       </c>
       <c r="H244" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I244" t="s">
         <v>2743</v>
@@ -26947,7 +26951,7 @@
         <v>2747</v>
       </c>
       <c r="N244" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O244" t="s">
         <v>2748</v>
@@ -26993,7 +26997,7 @@
         <v>27</v>
       </c>
       <c r="H245" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I245" t="s">
         <v>2753</v>
@@ -27011,7 +27015,7 @@
         <v>2757</v>
       </c>
       <c r="N245" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O245" t="s">
         <v>2758</v>
@@ -27075,7 +27079,7 @@
         <v>2765</v>
       </c>
       <c r="N246" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O246" t="s">
         <v>2766</v>
@@ -27121,7 +27125,7 @@
         <v>27</v>
       </c>
       <c r="H247" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I247" t="s">
         <v>2773</v>
@@ -27137,7 +27141,7 @@
         <v>2776</v>
       </c>
       <c r="N247" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O247" t="s">
         <v>2777</v>
@@ -27199,7 +27203,7 @@
         <v>2784</v>
       </c>
       <c r="N248" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O248" t="s">
         <v>2785</v>
@@ -27261,7 +27265,7 @@
         <v>2794</v>
       </c>
       <c r="N249" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O249" t="s">
         <v>2795</v>
@@ -27305,7 +27309,7 @@
         <v>27</v>
       </c>
       <c r="H250" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I250" t="s">
         <v>2799</v>
@@ -27323,7 +27327,7 @@
         <v>2803</v>
       </c>
       <c r="N250" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O250" t="s">
         <v>2804</v>
@@ -27385,7 +27389,7 @@
         <v>2816</v>
       </c>
       <c r="N251" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O251" t="s">
         <v>2817</v>
@@ -27431,7 +27435,7 @@
         <v>164</v>
       </c>
       <c r="H252" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I252" t="s">
         <v>2825</v>
@@ -27449,7 +27453,7 @@
         <v>2829</v>
       </c>
       <c r="N252" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O252" t="s">
         <v>2830</v>
@@ -27513,7 +27517,7 @@
         <v>2838</v>
       </c>
       <c r="N253" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O253" t="s">
         <v>2839</v>
@@ -27577,7 +27581,7 @@
         <v>2847</v>
       </c>
       <c r="N254" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O254" t="s">
         <v>2848</v>
@@ -27623,7 +27627,7 @@
         <v>27</v>
       </c>
       <c r="H255" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I255" t="s">
         <v>2854</v>
@@ -27641,7 +27645,7 @@
         <v>2858</v>
       </c>
       <c r="N255" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O255" t="s">
         <v>2859</v>
@@ -27687,7 +27691,7 @@
         <v>27</v>
       </c>
       <c r="H256" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I256" t="s">
         <v>2862</v>
@@ -27705,7 +27709,7 @@
         <v>2866</v>
       </c>
       <c r="N256" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O256" t="s">
         <v>2867</v>
@@ -27751,7 +27755,7 @@
         <v>27</v>
       </c>
       <c r="H257" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I257" t="s">
         <v>2871</v>
@@ -27769,7 +27773,7 @@
         <v>2875</v>
       </c>
       <c r="N257" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O257" t="s">
         <v>2876</v>
@@ -27833,7 +27837,7 @@
         <v>2888</v>
       </c>
       <c r="N258" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O258" t="s">
         <v>2889</v>
@@ -27897,7 +27901,7 @@
         <v>2899</v>
       </c>
       <c r="N259" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O259" t="s">
         <v>2900</v>
@@ -27943,7 +27947,7 @@
         <v>27</v>
       </c>
       <c r="H260" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I260" t="s">
         <v>2908</v>
@@ -27961,7 +27965,7 @@
         <v>2912</v>
       </c>
       <c r="N260" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O260" t="s">
         <v>2913</v>
@@ -28007,7 +28011,7 @@
         <v>27</v>
       </c>
       <c r="H261" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I261" t="s">
         <v>2920</v>
@@ -28025,7 +28029,7 @@
         <v>2924</v>
       </c>
       <c r="N261" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O261" t="s">
         <v>2925</v>
@@ -28071,7 +28075,7 @@
         <v>27</v>
       </c>
       <c r="H262" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I262" t="s">
         <v>2928</v>
@@ -28087,7 +28091,7 @@
         <v>2931</v>
       </c>
       <c r="N262" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O262" t="s">
         <v>2932</v>
@@ -28133,7 +28137,7 @@
         <v>27</v>
       </c>
       <c r="H263" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I263" t="s">
         <v>2939</v>
@@ -28151,7 +28155,7 @@
         <v>2943</v>
       </c>
       <c r="N263" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O263" t="s">
         <v>2944</v>
@@ -28195,7 +28199,7 @@
         <v>27</v>
       </c>
       <c r="H264" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I264" t="s">
         <v>2951</v>
@@ -28213,7 +28217,7 @@
         <v>2955</v>
       </c>
       <c r="N264" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O264" t="s">
         <v>2956</v>
@@ -28257,7 +28261,7 @@
         <v>27</v>
       </c>
       <c r="H265" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I265" t="s">
         <v>2960</v>
@@ -28275,7 +28279,7 @@
         <v>2964</v>
       </c>
       <c r="N265" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O265" t="s">
         <v>2965</v>
@@ -28319,7 +28323,7 @@
         <v>27</v>
       </c>
       <c r="H266" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I266" t="s">
         <v>2968</v>
@@ -28337,7 +28341,7 @@
         <v>2972</v>
       </c>
       <c r="N266" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O266" t="s">
         <v>2973</v>
@@ -28381,7 +28385,7 @@
         <v>27</v>
       </c>
       <c r="H267" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I267" t="s">
         <v>2976</v>
@@ -28399,7 +28403,7 @@
         <v>2980</v>
       </c>
       <c r="N267" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O267" t="s">
         <v>2981</v>
@@ -28443,7 +28447,7 @@
         <v>27</v>
       </c>
       <c r="H268" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I268" t="s">
         <v>2986</v>
@@ -28461,7 +28465,7 @@
         <v>2990</v>
       </c>
       <c r="N268" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O268" t="s">
         <v>2991</v>
@@ -28507,7 +28511,7 @@
         <v>27</v>
       </c>
       <c r="H269" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I269" t="s">
         <v>2999</v>
@@ -28525,7 +28529,7 @@
         <v>3003</v>
       </c>
       <c r="N269" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O269" t="s">
         <v>3004</v>
@@ -28589,7 +28593,7 @@
         <v>3013</v>
       </c>
       <c r="N270" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O270" t="s">
         <v>3014</v>
@@ -28651,7 +28655,7 @@
         <v>3024</v>
       </c>
       <c r="N271" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O271" t="s">
         <v>3025</v>
@@ -28697,7 +28701,7 @@
         <v>27</v>
       </c>
       <c r="H272" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I272" t="s">
         <v>3034</v>
@@ -28715,7 +28719,7 @@
         <v>3038</v>
       </c>
       <c r="N272" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O272" t="s">
         <v>3039</v>
@@ -28779,7 +28783,7 @@
         <v>3051</v>
       </c>
       <c r="N273" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O273" t="s">
         <v>3052</v>
@@ -28843,7 +28847,7 @@
         <v>3062</v>
       </c>
       <c r="N274" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O274" t="s">
         <v>3063</v>
@@ -28889,7 +28893,7 @@
         <v>27</v>
       </c>
       <c r="H275" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I275" t="s">
         <v>3066</v>
@@ -28907,7 +28911,7 @@
         <v>3070</v>
       </c>
       <c r="N275" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O275" t="s">
         <v>3071</v>
@@ -28971,7 +28975,7 @@
         <v>3081</v>
       </c>
       <c r="N276" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O276" t="s">
         <v>3082</v>
@@ -29017,7 +29021,7 @@
         <v>27</v>
       </c>
       <c r="H277" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I277" t="s">
         <v>3088</v>
@@ -29035,7 +29039,7 @@
         <v>3092</v>
       </c>
       <c r="N277" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O277" t="s">
         <v>3093</v>
@@ -29099,7 +29103,7 @@
         <v>3103</v>
       </c>
       <c r="N278" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O278" t="s">
         <v>3104</v>
@@ -29163,7 +29167,7 @@
         <v>3111</v>
       </c>
       <c r="N279" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O279" t="s">
         <v>3112</v>
@@ -29227,7 +29231,7 @@
         <v>3120</v>
       </c>
       <c r="N280" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O280" t="s">
         <v>3121</v>
@@ -29291,7 +29295,7 @@
         <v>3129</v>
       </c>
       <c r="N281" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O281" t="s">
         <v>3130</v>
@@ -29353,7 +29357,7 @@
         <v>3137</v>
       </c>
       <c r="N282" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O282" t="s">
         <v>3138</v>
@@ -29399,7 +29403,7 @@
         <v>27</v>
       </c>
       <c r="H283" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I283" t="s">
         <v>3145</v>
@@ -29415,7 +29419,7 @@
         <v>3148</v>
       </c>
       <c r="N283" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O283" t="s">
         <v>3149</v>
@@ -29479,7 +29483,7 @@
         <v>3157</v>
       </c>
       <c r="N284" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O284" t="s">
         <v>3158</v>
@@ -29523,7 +29527,7 @@
         <v>27</v>
       </c>
       <c r="H285" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I285" t="s">
         <v>3165</v>
@@ -29541,7 +29545,7 @@
         <v>3169</v>
       </c>
       <c r="N285" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O285" t="s">
         <v>3170</v>
@@ -29585,7 +29589,7 @@
         <v>27</v>
       </c>
       <c r="H286" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I286" t="s">
         <v>3173</v>
@@ -29603,7 +29607,7 @@
         <v>3177</v>
       </c>
       <c r="N286" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O286" t="s">
         <v>3178</v>
@@ -29647,7 +29651,7 @@
         <v>27</v>
       </c>
       <c r="H287" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I287" t="s">
         <v>3181</v>
@@ -29665,7 +29669,7 @@
         <v>3185</v>
       </c>
       <c r="N287" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O287" t="s">
         <v>3186</v>
@@ -29711,7 +29715,7 @@
         <v>27</v>
       </c>
       <c r="H288" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I288" t="s">
         <v>3189</v>
@@ -29729,7 +29733,7 @@
         <v>3193</v>
       </c>
       <c r="N288" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O288" t="s">
         <v>3194</v>
@@ -29773,7 +29777,7 @@
         <v>27</v>
       </c>
       <c r="H289" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I289" t="s">
         <v>3201</v>
@@ -29791,7 +29795,7 @@
         <v>3205</v>
       </c>
       <c r="N289" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O289" t="s">
         <v>3206</v>
@@ -29855,7 +29859,7 @@
         <v>3215</v>
       </c>
       <c r="N290" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O290" t="s">
         <v>3216</v>
@@ -29901,7 +29905,7 @@
         <v>27</v>
       </c>
       <c r="H291" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I291" t="s">
         <v>3222</v>
@@ -29917,7 +29921,7 @@
         <v>3225</v>
       </c>
       <c r="N291" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O291" t="s">
         <v>3226</v>
@@ -29963,7 +29967,7 @@
         <v>27</v>
       </c>
       <c r="H292" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I292" t="s">
         <v>3231</v>
@@ -29981,7 +29985,7 @@
         <v>3235</v>
       </c>
       <c r="N292" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O292" t="s">
         <v>3236</v>
@@ -30045,7 +30049,7 @@
         <v>3244</v>
       </c>
       <c r="N293" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O293" t="s">
         <v>3245</v>
@@ -30091,7 +30095,7 @@
         <v>27</v>
       </c>
       <c r="H294" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I294" t="s">
         <v>3250</v>
@@ -30109,7 +30113,7 @@
         <v>3254</v>
       </c>
       <c r="N294" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O294" t="s">
         <v>3255</v>
@@ -30173,7 +30177,7 @@
         <v>3265</v>
       </c>
       <c r="N295" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O295" t="s">
         <v>3266</v>
@@ -30237,7 +30241,7 @@
         <v>3277</v>
       </c>
       <c r="N296" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O296" t="s">
         <v>3278</v>
@@ -30299,7 +30303,7 @@
         <v>3286</v>
       </c>
       <c r="N297" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O297" t="s">
         <v>3287</v>
@@ -30361,7 +30365,7 @@
         <v>3298</v>
       </c>
       <c r="N298" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O298" t="s">
         <v>3299</v>
@@ -30425,7 +30429,7 @@
         <v>3310</v>
       </c>
       <c r="N299" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O299" t="s">
         <v>3311</v>
@@ -30489,7 +30493,7 @@
         <v>3319</v>
       </c>
       <c r="N300" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O300" t="s">
         <v>3320</v>
@@ -30553,7 +30557,7 @@
         <v>3329</v>
       </c>
       <c r="N301" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O301" t="s">
         <v>3330</v>
@@ -30599,7 +30603,7 @@
         <v>27</v>
       </c>
       <c r="H302" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I302" t="s">
         <v>3338</v>
@@ -30617,7 +30621,7 @@
         <v>3342</v>
       </c>
       <c r="N302" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O302" t="s">
         <v>3343</v>
@@ -30663,7 +30667,7 @@
         <v>27</v>
       </c>
       <c r="H303" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I303" t="s">
         <v>3350</v>
@@ -30681,7 +30685,7 @@
         <v>3354</v>
       </c>
       <c r="N303" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O303" t="s">
         <v>3355</v>
@@ -30745,7 +30749,7 @@
         <v>3366</v>
       </c>
       <c r="N304" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O304" t="s">
         <v>3367</v>
@@ -30809,7 +30813,7 @@
         <v>3375</v>
       </c>
       <c r="N305" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O305" t="s">
         <v>3376</v>
@@ -30873,7 +30877,7 @@
         <v>3384</v>
       </c>
       <c r="N306" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O306" t="s">
         <v>3385</v>
@@ -30937,7 +30941,7 @@
         <v>3396</v>
       </c>
       <c r="N307" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O307" t="s">
         <v>3397</v>
@@ -30999,7 +31003,7 @@
         <v>3404</v>
       </c>
       <c r="N308" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O308" t="s">
         <v>3405</v>
@@ -31061,7 +31065,7 @@
         <v>3412</v>
       </c>
       <c r="N309" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O309" t="s">
         <v>3413</v>
@@ -31125,7 +31129,7 @@
         <v>3421</v>
       </c>
       <c r="N310" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O310" t="s">
         <v>3422</v>
@@ -31189,7 +31193,7 @@
         <v>3434</v>
       </c>
       <c r="N311" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O311" t="s">
         <v>3435</v>
@@ -31235,7 +31239,7 @@
         <v>27</v>
       </c>
       <c r="H312" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I312" t="s">
         <v>3443</v>
@@ -31253,7 +31257,7 @@
         <v>3447</v>
       </c>
       <c r="N312" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O312" t="s">
         <v>3448</v>
@@ -31317,7 +31321,7 @@
         <v>3457</v>
       </c>
       <c r="N313" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O313" t="s">
         <v>3458</v>
@@ -31381,7 +31385,7 @@
         <v>3466</v>
       </c>
       <c r="N314" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O314" t="s">
         <v>3467</v>
@@ -31445,7 +31449,7 @@
         <v>3475</v>
       </c>
       <c r="N315" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O315" t="s">
         <v>3476</v>
@@ -31491,7 +31495,7 @@
         <v>164</v>
       </c>
       <c r="H316" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I316" t="s">
         <v>3482</v>
@@ -31509,7 +31513,7 @@
         <v>3486</v>
       </c>
       <c r="N316" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O316" t="s">
         <v>3487</v>
@@ -31573,7 +31577,7 @@
         <v>3497</v>
       </c>
       <c r="N317" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O317" t="s">
         <v>3498</v>
@@ -31637,7 +31641,7 @@
         <v>3509</v>
       </c>
       <c r="N318" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O318" t="s">
         <v>3510</v>
@@ -31701,7 +31705,7 @@
         <v>3519</v>
       </c>
       <c r="N319" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O319" t="s">
         <v>3520</v>
@@ -31765,7 +31769,7 @@
         <v>3528</v>
       </c>
       <c r="N320" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O320" t="s">
         <v>3529</v>
@@ -31829,7 +31833,7 @@
         <v>3537</v>
       </c>
       <c r="N321" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O321" t="s">
         <v>3538</v>
@@ -31875,7 +31879,7 @@
         <v>27</v>
       </c>
       <c r="H322" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I322" t="s">
         <v>3542</v>
@@ -31893,7 +31897,7 @@
         <v>3546</v>
       </c>
       <c r="N322" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O322" t="s">
         <v>3547</v>
@@ -31957,7 +31961,7 @@
         <v>3557</v>
       </c>
       <c r="N323" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O323" t="s">
         <v>3558</v>
@@ -32021,7 +32025,7 @@
         <v>3565</v>
       </c>
       <c r="N324" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O324" t="s">
         <v>3566</v>
@@ -32085,7 +32089,7 @@
         <v>3574</v>
       </c>
       <c r="N325" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="O325" t="s">
         <v>3575</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-03-17
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -11233,9 +11233,7 @@
       <c r="R2" t="s">
         <v>37</v>
       </c>
-      <c r="S2" t="s">
-        <v>37</v>
-      </c>
+      <c r="S2"/>
       <c r="T2" t="s">
         <v>38</v>
       </c>
@@ -11299,9 +11297,7 @@
       <c r="R3" t="s">
         <v>37</v>
       </c>
-      <c r="S3" t="s">
-        <v>37</v>
-      </c>
+      <c r="S3"/>
       <c r="T3" t="s">
         <v>52</v>
       </c>

</xml_diff>

<commit_message>
Update parliament data - 2026-04-08
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -16724,9 +16724,7 @@
       <c r="D85" t="s">
         <v>1001</v>
       </c>
-      <c r="E85" t="s">
-        <v>44</v>
-      </c>
+      <c r="E85"/>
       <c r="F85" t="s">
         <v>1002</v>
       </c>

</xml_diff>

<commit_message>
Update parliament data - 2026-05-06
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -185,6 +185,57 @@
     <t xml:space="preserve">Scienza e ricerca|Ambiente|Salute</t>
   </si>
   <si>
+    <t xml:space="preserve">26.3398</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gredig Corina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pvl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EFD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einführung eines öffentlichen Registers der Subventionsempfänger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Créer un registre public des bénéficiaires de subventions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Introduzione di un registro pubblico dei beneficiari di sussidi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de créer un registre central public des bénéficiaires de subventions fédérales. Ce registre sera conçu pour compléter la banque de données sur les subventions et sa tenue sera confiée à la Confédération ou au Contrôle fédéral des finances. Il indiquera au minimum le nom du bénéficiaire ou son type, la nature et l’objet de la subvention, le montant annuel versé et l’office fédéral compétent et utilisera les données dont disposent les offices fédéraux.&amp;nbsp;&lt;br&gt;Les restrictions dictées par la protection des données et par la sécurité seront réservées.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, ein öffentlich einsehbares, zentrales Register der &amp;nbsp;Empfängerinnen und Empfänger von Bundessubventionen einzuführen. Das Register soll als Ergänzung zur bestehenden Subventionsdatenbank ausgestaltet und durch Bund oder EFK geführt werden. Es hat mindestens den Namen oder Empfängertyp, Art und Zweck der Subvention, den jährlich ausbezahlten Betrag sowie das zuständige Bundesamt auszuweisen. Es soll bestehenden Daten der Bundesämter nutzen.&amp;nbsp;&lt;br&gt;Datenschutz- und sicherheitsrelevante Einschränkungen bleiben vorbehalten.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eingereicht / Déposé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263398</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263398</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Staatspolitik|Finanzwesen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politique d'Etat|Finances</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Politica nazionale|Finanze</t>
+  </si>
+  <si>
     <t xml:space="preserve">26.3485</t>
   </si>
   <si>
@@ -197,12 +248,6 @@
     <t xml:space="preserve">UDC</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EFD</t>
-  </si>
-  <si>
     <t xml:space="preserve">Externes Audit des Bundesamts für Zoll und Grenzsicherheit zur Wiederherstellung des Vertrauens des Personals und der Wirtschaft</t>
   </si>
   <si>
@@ -218,9 +263,6 @@
     <t xml:space="preserve">&lt;p&gt;Bevor irreversible Entscheide getroffen werden, wird der Bundesrat beauftragt, ein externes Audit des Bundesamts für Zoll und Grenzsicherheit (BAZG) und dessen laufender Umstrukturierung in Auftrag zu geben, das insbesondere folgende Punkte umfasst:&lt;/p&gt;&lt;p&gt;&amp;nbsp;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Angemessenheit der Mittel (Budget und Personal) für die vielfältigen Aufgaben des BAZG, insbesondere für die Überwachung der Landesgrenze, die Migrationskontrolle und die Bekämpfung von Schmuggel aller Art (landwirtschaftliche Produkte, Tiere, invasive Pflanzen);&lt;/li&gt;&lt;li&gt;Wirksamkeit des Programms Dazit bei der Zollerhebung (rückläufige Einnahmen&amp;nbsp;2025), insbesondere angesichts des Wegfalls der systematischen Kontrolle ausländischer Lastwagen und der Erwartungen der Wirtschaft (in Anlehnung an die sehr harte Kritik des Transportunternehmers Marco Tepoorten, der von einer «systemischen Desorganisation» sprach);&lt;/li&gt;&lt;li&gt;Flexibilisierung von Allegra;&lt;/li&gt;&lt;li&gt;Krankheitsabsenzen und Abgänge beim BAZG;&lt;/li&gt;&lt;li&gt;Attraktivität des BAZG-Personalstatus;&lt;/li&gt;&lt;li&gt;Ausbildung (mit offenbar ungewöhnlich hoher Durchfallquote);&lt;/li&gt;&lt;li&gt;untypische Fluktuationsrate bei den Führungskräften des BAZG;&lt;/li&gt;&lt;li&gt;Wäre es nicht angebracht, Lehren aus vergleichbaren Umstrukturierungen im Ausland (Österreich, Kanada) zu ziehen – insbesondere aus gewissen Misserfolgen –, bevor weiter in eine fragwürdige Richtung vorgeprescht wird?&lt;/li&gt;&lt;li&gt;Welche Massnahmen sind notwendig, um das Vertrauen des Personals und der Wirtschaft wiederherzustellen und die Wirksamkeit des BAZG bei der Aufgabenerfüllung zu gewährleisten?&lt;/li&gt;&lt;/ul&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">Eingereicht / Déposé</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263485</t>
   </si>
   <si>
@@ -234,48 +276,6 @@
   </si>
   <si>
     <t xml:space="preserve">Politica nazionale|Finanze|Occupazione e lavoro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.3398</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gredig Corina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pvl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Einführung eines öffentlichen Registers der Subventionsempfänger</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Créer un registre public des bénéficiaires de subventions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Introduzione di un registro pubblico dei beneficiari di sussidi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de créer un registre central public des bénéficiaires de subventions fédérales. Ce registre sera conçu pour compléter la banque de données sur les subventions et sa tenue sera confiée à la Confédération ou au Contrôle fédéral des finances. Il indiquera au minimum le nom du bénéficiaire ou son type, la nature et l’objet de la subvention, le montant annuel versé et l’office fédéral compétent et utilisera les données dont disposent les offices fédéraux.&amp;nbsp;&lt;br&gt;Les restrictions dictées par la protection des données et par la sécurité seront réservées.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, ein öffentlich einsehbares, zentrales Register der &amp;nbsp;Empfängerinnen und Empfänger von Bundessubventionen einzuführen. Das Register soll als Ergänzung zur bestehenden Subventionsdatenbank ausgestaltet und durch Bund oder EFK geführt werden. Es hat mindestens den Namen oder Empfängertyp, Art und Zweck der Subvention, den jährlich ausbezahlten Betrag sowie das zuständige Bundesamt auszuweisen. Es soll bestehenden Daten der Bundesämter nutzen.&amp;nbsp;&lt;br&gt;Datenschutz- und sicherheitsrelevante Einschränkungen bleiben vorbehalten.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263398</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263398</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Staatspolitik|Finanzwesen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politique d'Etat|Finances</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Politica nazionale|Finanze</t>
   </si>
   <si>
     <t xml:space="preserve">26.3487</t>
@@ -11473,7 +11473,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>20263485</v>
+        <v>20263398</v>
       </c>
       <c r="B4" t="s">
         <v>57</v>
@@ -11539,7 +11539,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>20263398</v>
+        <v>20263485</v>
       </c>
       <c r="B5" t="s">
         <v>74</v>
@@ -11749,7 +11749,7 @@
         <v>120</v>
       </c>
       <c r="E8" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F8" t="s">
         <v>121</v>
@@ -12007,7 +12007,7 @@
         <v>172</v>
       </c>
       <c r="C12" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D12" t="s">
         <v>173</v>
@@ -12269,7 +12269,7 @@
         <v>225</v>
       </c>
       <c r="E16" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F16" t="s">
         <v>226</v>
@@ -12312,13 +12312,13 @@
       </c>
       <c r="S16"/>
       <c r="T16" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U16" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V16" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17">
@@ -12335,7 +12335,7 @@
         <v>237</v>
       </c>
       <c r="E17" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F17" t="s">
         <v>238</v>
@@ -12395,7 +12395,7 @@
         <v>251</v>
       </c>
       <c r="C18" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D18" t="s">
         <v>252</v>
@@ -12527,7 +12527,7 @@
         <v>276</v>
       </c>
       <c r="C20" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D20" t="s">
         <v>277</v>
@@ -12599,7 +12599,7 @@
         <v>283</v>
       </c>
       <c r="E21" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F21" t="s">
         <v>238</v>
@@ -12725,7 +12725,7 @@
         <v>307</v>
       </c>
       <c r="C23" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D23" t="s">
         <v>133</v>
@@ -12791,7 +12791,7 @@
         <v>318</v>
       </c>
       <c r="C24" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D24" t="s">
         <v>319</v>
@@ -12923,7 +12923,7 @@
         <v>344</v>
       </c>
       <c r="C26" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D26" t="s">
         <v>345</v>
@@ -12995,7 +12995,7 @@
         <v>357</v>
       </c>
       <c r="E27" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F27" t="s">
         <v>358</v>
@@ -13059,7 +13059,7 @@
         <v>369</v>
       </c>
       <c r="E28" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F28" t="s">
         <v>358</v>
@@ -13185,7 +13185,7 @@
         <v>394</v>
       </c>
       <c r="C30" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D30" t="s">
         <v>395</v>
@@ -13251,7 +13251,7 @@
         <v>407</v>
       </c>
       <c r="C31" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D31" t="s">
         <v>43</v>
@@ -13383,7 +13383,7 @@
         <v>432</v>
       </c>
       <c r="C33" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D33" t="s">
         <v>433</v>
@@ -13449,13 +13449,13 @@
         <v>445</v>
       </c>
       <c r="C34" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D34" t="s">
         <v>446</v>
       </c>
       <c r="E34" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F34" t="s">
         <v>409</v>
@@ -13975,7 +13975,7 @@
         <v>539</v>
       </c>
       <c r="C42" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D42" t="s">
         <v>540</v>
@@ -14305,7 +14305,7 @@
         <v>597</v>
       </c>
       <c r="E47" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F47" t="s">
         <v>584</v>
@@ -14363,7 +14363,7 @@
         <v>607</v>
       </c>
       <c r="C48" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D48" t="s">
         <v>608</v>
@@ -14761,7 +14761,7 @@
         <v>446</v>
       </c>
       <c r="E54" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F54" t="s">
         <v>680</v>
@@ -14953,7 +14953,7 @@
         <v>709</v>
       </c>
       <c r="C57" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D57" t="s">
         <v>43</v>
@@ -15019,7 +15019,7 @@
         <v>720</v>
       </c>
       <c r="C58" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D58" t="s">
         <v>43</v>
@@ -15287,7 +15287,7 @@
         <v>446</v>
       </c>
       <c r="E62" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F62" t="s">
         <v>751</v>
@@ -15479,7 +15479,7 @@
         <v>794</v>
       </c>
       <c r="E65" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F65" t="s">
         <v>795</v>
@@ -15739,7 +15739,7 @@
         <v>830</v>
       </c>
       <c r="E69" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F69" t="s">
         <v>821</v>
@@ -15799,13 +15799,13 @@
         <v>841</v>
       </c>
       <c r="C70" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D70" t="s">
         <v>830</v>
       </c>
       <c r="E70" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F70" t="s">
         <v>821</v>
@@ -15997,7 +15997,7 @@
         <v>871</v>
       </c>
       <c r="C73" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D73" t="s">
         <v>872</v>
@@ -16061,7 +16061,7 @@
         <v>881</v>
       </c>
       <c r="C74" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D74" t="s">
         <v>882</v>
@@ -16128,10 +16128,10 @@
         <v>23</v>
       </c>
       <c r="D75" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="E75" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F75" t="s">
         <v>893</v>
@@ -16191,13 +16191,13 @@
         <v>904</v>
       </c>
       <c r="C76" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D76" t="s">
         <v>446</v>
       </c>
       <c r="E76" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F76" t="s">
         <v>905</v>
@@ -16323,13 +16323,13 @@
         <v>924</v>
       </c>
       <c r="C78" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D78" t="s">
         <v>925</v>
       </c>
       <c r="E78" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F78" t="s">
         <v>926</v>
@@ -16500,13 +16500,13 @@
       </c>
       <c r="S80"/>
       <c r="T80" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U80" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V80" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="81">
@@ -16655,7 +16655,7 @@
         <v>980</v>
       </c>
       <c r="E83" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F83" t="s">
         <v>981</v>
@@ -16721,7 +16721,7 @@
         <v>993</v>
       </c>
       <c r="E84" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F84" t="s">
         <v>994</v>
@@ -16781,7 +16781,7 @@
         <v>1005</v>
       </c>
       <c r="C85" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D85" t="s">
         <v>1006</v>
@@ -16851,7 +16851,7 @@
         <v>1019</v>
       </c>
       <c r="E86" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F86" t="s">
         <v>1020</v>
@@ -16969,13 +16969,13 @@
         <v>1039</v>
       </c>
       <c r="C88" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D88" t="s">
         <v>597</v>
       </c>
       <c r="E88" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F88" t="s">
         <v>1040</v>
@@ -17167,7 +17167,7 @@
         <v>1069</v>
       </c>
       <c r="C91" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D91" t="s">
         <v>1070</v>
@@ -17233,13 +17233,13 @@
         <v>1082</v>
       </c>
       <c r="C92" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D92" t="s">
         <v>1083</v>
       </c>
       <c r="E92" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F92" t="s">
         <v>1071</v>
@@ -17299,7 +17299,7 @@
         <v>1094</v>
       </c>
       <c r="C93" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D93" t="s">
         <v>43</v>
@@ -17348,13 +17348,13 @@
       </c>
       <c r="S93"/>
       <c r="T93" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U93" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V93" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="94">
@@ -17365,7 +17365,7 @@
         <v>1103</v>
       </c>
       <c r="C94" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D94" t="s">
         <v>1104</v>
@@ -17497,7 +17497,7 @@
         <v>1126</v>
       </c>
       <c r="C96" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D96" t="s">
         <v>1127</v>
@@ -17701,7 +17701,7 @@
         <v>1164</v>
       </c>
       <c r="E99" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F99" t="s">
         <v>1152</v>
@@ -17893,7 +17893,7 @@
         <v>1192</v>
       </c>
       <c r="C102" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D102" t="s">
         <v>1193</v>
@@ -17959,7 +17959,7 @@
         <v>1205</v>
       </c>
       <c r="C103" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D103" t="s">
         <v>213</v>
@@ -18025,7 +18025,7 @@
         <v>1217</v>
       </c>
       <c r="C104" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D104" t="s">
         <v>213</v>
@@ -18163,7 +18163,7 @@
         <v>830</v>
       </c>
       <c r="E106" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F106" t="s">
         <v>1230</v>
@@ -18223,13 +18223,13 @@
         <v>1252</v>
       </c>
       <c r="C107" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D107" t="s">
         <v>446</v>
       </c>
       <c r="E107" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F107" t="s">
         <v>1230</v>
@@ -18272,13 +18272,13 @@
       </c>
       <c r="S107"/>
       <c r="T107" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U107" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V107" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="108">
@@ -18355,7 +18355,7 @@
         <v>1273</v>
       </c>
       <c r="C109" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D109" t="s">
         <v>967</v>
@@ -18553,13 +18553,13 @@
         <v>1301</v>
       </c>
       <c r="C112" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D112" t="s">
         <v>1302</v>
       </c>
       <c r="E112" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F112" t="s">
         <v>1293</v>
@@ -19011,13 +19011,13 @@
         <v>1374</v>
       </c>
       <c r="C119" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D119" t="s">
         <v>1375</v>
       </c>
       <c r="E119" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F119" t="s">
         <v>1376</v>
@@ -19077,7 +19077,7 @@
         <v>1387</v>
       </c>
       <c r="C120" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D120" t="s">
         <v>1388</v>
@@ -19211,7 +19211,7 @@
         <v>1409</v>
       </c>
       <c r="E122" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F122" t="s">
         <v>1410</v>
@@ -19269,7 +19269,7 @@
         <v>1417</v>
       </c>
       <c r="C123" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D123" t="s">
         <v>1418</v>
@@ -19601,7 +19601,7 @@
         <v>1480</v>
       </c>
       <c r="E128" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F128" t="s">
         <v>1481</v>
@@ -19989,7 +19989,7 @@
         <v>1550</v>
       </c>
       <c r="C134" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D134" t="s">
         <v>1551</v>
@@ -20061,7 +20061,7 @@
         <v>1564</v>
       </c>
       <c r="E135" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F135" t="s">
         <v>1552</v>
@@ -20125,7 +20125,7 @@
         <v>120</v>
       </c>
       <c r="E136" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F136" t="s">
         <v>1575</v>
@@ -20183,7 +20183,7 @@
         <v>1582</v>
       </c>
       <c r="C137" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D137" t="s">
         <v>872</v>
@@ -20313,7 +20313,7 @@
         <v>1604</v>
       </c>
       <c r="C139" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D139" t="s">
         <v>967</v>
@@ -20379,13 +20379,13 @@
         <v>1616</v>
       </c>
       <c r="C140" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D140" t="s">
         <v>1480</v>
       </c>
       <c r="E140" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F140" t="s">
         <v>1605</v>
@@ -20451,7 +20451,7 @@
         <v>1628</v>
       </c>
       <c r="E141" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F141" t="s">
         <v>1605</v>
@@ -20511,13 +20511,13 @@
         <v>1639</v>
       </c>
       <c r="C142" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D142" t="s">
         <v>1640</v>
       </c>
       <c r="E142" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F142" t="s">
         <v>1641</v>
@@ -20649,7 +20649,7 @@
         <v>1302</v>
       </c>
       <c r="E144" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F144" t="s">
         <v>1665</v>
@@ -20969,7 +20969,7 @@
         <v>1710</v>
       </c>
       <c r="C149" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D149" t="s">
         <v>1711</v>
@@ -21035,7 +21035,7 @@
         <v>1722</v>
       </c>
       <c r="C150" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D150" t="s">
         <v>43</v>
@@ -21299,7 +21299,7 @@
         <v>1766</v>
       </c>
       <c r="C154" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D154" t="s">
         <v>1767</v>
@@ -21623,7 +21623,7 @@
         <v>1814</v>
       </c>
       <c r="C159" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D159" t="s">
         <v>1815</v>
@@ -21687,7 +21687,7 @@
         <v>1825</v>
       </c>
       <c r="C160" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D160" t="s">
         <v>608</v>
@@ -21817,7 +21817,7 @@
         <v>1849</v>
       </c>
       <c r="C162" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D162" t="s">
         <v>1104</v>
@@ -21883,7 +21883,7 @@
         <v>1861</v>
       </c>
       <c r="C163" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D163" t="s">
         <v>1862</v>
@@ -22085,7 +22085,7 @@
         <v>1897</v>
       </c>
       <c r="E166" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F166" t="s">
         <v>1885</v>
@@ -22145,7 +22145,7 @@
         <v>1908</v>
       </c>
       <c r="C167" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D167" t="s">
         <v>1909</v>
@@ -22283,7 +22283,7 @@
         <v>830</v>
       </c>
       <c r="E169" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F169" t="s">
         <v>1921</v>
@@ -22343,7 +22343,7 @@
         <v>1943</v>
       </c>
       <c r="C170" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D170" t="s">
         <v>862</v>
@@ -22481,7 +22481,7 @@
         <v>1961</v>
       </c>
       <c r="E172" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F172" t="s">
         <v>1962</v>
@@ -22607,7 +22607,7 @@
         <v>1985</v>
       </c>
       <c r="C174" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D174" t="s">
         <v>1986</v>
@@ -22739,7 +22739,7 @@
         <v>2003</v>
       </c>
       <c r="C176" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D176" t="s">
         <v>2004</v>
@@ -23329,7 +23329,7 @@
         <v>2105</v>
       </c>
       <c r="C185" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D185" t="s">
         <v>1397</v>
@@ -23593,13 +23593,13 @@
         <v>2151</v>
       </c>
       <c r="C189" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D189" t="s">
         <v>2152</v>
       </c>
       <c r="E189" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F189" t="s">
         <v>2153</v>
@@ -23795,7 +23795,7 @@
         <v>1628</v>
       </c>
       <c r="E192" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F192" t="s">
         <v>2189</v>
@@ -23855,7 +23855,7 @@
         <v>2197</v>
       </c>
       <c r="C193" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D193" t="s">
         <v>608</v>
@@ -24115,13 +24115,13 @@
         <v>2246</v>
       </c>
       <c r="C197" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D197" t="s">
         <v>446</v>
       </c>
       <c r="E197" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F197" t="s">
         <v>2247</v>
@@ -24181,7 +24181,7 @@
         <v>2258</v>
       </c>
       <c r="C198" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D198" t="s">
         <v>2259</v>
@@ -24245,7 +24245,7 @@
         <v>2271</v>
       </c>
       <c r="C199" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D199" t="s">
         <v>2272</v>
@@ -24309,7 +24309,7 @@
         <v>2284</v>
       </c>
       <c r="C200" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D200" t="s">
         <v>2272</v>
@@ -24373,13 +24373,13 @@
         <v>2295</v>
       </c>
       <c r="C201" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D201" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="E201" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F201" t="s">
         <v>226</v>
@@ -24443,7 +24443,7 @@
         <v>830</v>
       </c>
       <c r="E202" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F202" t="s">
         <v>226</v>
@@ -24501,7 +24501,7 @@
         <v>2314</v>
       </c>
       <c r="C203" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D203" t="s">
         <v>2315</v>
@@ -24565,7 +24565,7 @@
         <v>2327</v>
       </c>
       <c r="C204" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D204" t="s">
         <v>484</v>
@@ -24635,7 +24635,7 @@
         <v>2339</v>
       </c>
       <c r="E205" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F205" t="s">
         <v>2340</v>
@@ -24753,7 +24753,7 @@
         <v>2357</v>
       </c>
       <c r="C207" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D207" t="s">
         <v>1057</v>
@@ -24800,13 +24800,13 @@
       <c r="R207"/>
       <c r="S207"/>
       <c r="T207" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U207" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V207" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="208">
@@ -24817,7 +24817,7 @@
         <v>2366</v>
       </c>
       <c r="C208" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D208" t="s">
         <v>2367</v>
@@ -24881,7 +24881,7 @@
         <v>2376</v>
       </c>
       <c r="C209" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D209" t="s">
         <v>188</v>
@@ -24945,7 +24945,7 @@
         <v>2387</v>
       </c>
       <c r="C210" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D210" t="s">
         <v>2388</v>
@@ -24992,13 +24992,13 @@
       <c r="R210"/>
       <c r="S210"/>
       <c r="T210" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U210" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V210" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="211">
@@ -25009,7 +25009,7 @@
         <v>2394</v>
       </c>
       <c r="C211" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D211" t="s">
         <v>2395</v>
@@ -25137,7 +25137,7 @@
         <v>2414</v>
       </c>
       <c r="C213" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D213" t="s">
         <v>2415</v>
@@ -25515,7 +25515,7 @@
         <v>2472</v>
       </c>
       <c r="C219" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D219" t="s">
         <v>2473</v>
@@ -25580,10 +25580,10 @@
         <v>187</v>
       </c>
       <c r="D220" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="E220" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F220" t="s">
         <v>174</v>
@@ -25827,7 +25827,7 @@
         <v>2521</v>
       </c>
       <c r="C224" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D224" t="s">
         <v>2522</v>
@@ -25889,7 +25889,7 @@
         <v>2531</v>
       </c>
       <c r="C225" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D225" t="s">
         <v>2532</v>
@@ -25959,7 +25959,7 @@
         <v>1302</v>
       </c>
       <c r="E226" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F226" t="s">
         <v>2545</v>
@@ -26023,7 +26023,7 @@
         <v>2557</v>
       </c>
       <c r="E227" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F227" t="s">
         <v>2558</v>
@@ -26149,7 +26149,7 @@
         <v>2578</v>
       </c>
       <c r="E229" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F229" t="s">
         <v>2579</v>
@@ -26210,10 +26210,10 @@
         <v>23</v>
       </c>
       <c r="D230" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="E230" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F230" t="s">
         <v>2579</v>
@@ -26341,7 +26341,7 @@
         <v>1628</v>
       </c>
       <c r="E232" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F232" t="s">
         <v>2611</v>
@@ -26655,7 +26655,7 @@
         <v>2658</v>
       </c>
       <c r="C237" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D237" t="s">
         <v>2659</v>
@@ -26851,7 +26851,7 @@
         <v>2695</v>
       </c>
       <c r="E240" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F240" t="s">
         <v>2696</v>
@@ -26909,13 +26909,13 @@
         <v>2707</v>
       </c>
       <c r="C241" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D241" t="s">
         <v>1302</v>
       </c>
       <c r="E241" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F241" t="s">
         <v>2696</v>
@@ -26979,7 +26979,7 @@
         <v>120</v>
       </c>
       <c r="E242" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F242" t="s">
         <v>2696</v>
@@ -27037,7 +27037,7 @@
         <v>2729</v>
       </c>
       <c r="C243" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D243" t="s">
         <v>2599</v>
@@ -27107,7 +27107,7 @@
         <v>2742</v>
       </c>
       <c r="E244" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F244" t="s">
         <v>2730</v>
@@ -27229,7 +27229,7 @@
         <v>2766</v>
       </c>
       <c r="C246" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D246" t="s">
         <v>2767</v>
@@ -27417,13 +27417,13 @@
         <v>2793</v>
       </c>
       <c r="C249" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D249" t="s">
         <v>2794</v>
       </c>
       <c r="E249" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F249" t="s">
         <v>2795</v>
@@ -27545,13 +27545,13 @@
         <v>2813</v>
       </c>
       <c r="C251" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D251" t="s">
         <v>120</v>
       </c>
       <c r="E251" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F251" t="s">
         <v>2805</v>
@@ -27615,7 +27615,7 @@
         <v>2794</v>
       </c>
       <c r="E252" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F252" t="s">
         <v>2825</v>
@@ -27919,7 +27919,7 @@
         <v>2875</v>
       </c>
       <c r="C257" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D257" t="s">
         <v>2876</v>
@@ -27983,7 +27983,7 @@
         <v>2885</v>
       </c>
       <c r="C258" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D258" t="s">
         <v>1711</v>
@@ -28111,7 +28111,7 @@
         <v>2906</v>
       </c>
       <c r="C260" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D260" t="s">
         <v>574</v>
@@ -28175,7 +28175,7 @@
         <v>2914</v>
       </c>
       <c r="C261" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D261" t="s">
         <v>574</v>
@@ -28239,13 +28239,13 @@
         <v>2922</v>
       </c>
       <c r="C262" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D262" t="s">
         <v>2923</v>
       </c>
       <c r="E262" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F262" t="s">
         <v>2886</v>
@@ -28373,7 +28373,7 @@
         <v>1019</v>
       </c>
       <c r="E264" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F264" t="s">
         <v>2936</v>
@@ -28437,7 +28437,7 @@
         <v>2959</v>
       </c>
       <c r="E265" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F265" t="s">
         <v>2960</v>
@@ -28495,7 +28495,7 @@
         <v>2971</v>
       </c>
       <c r="C266" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D266" t="s">
         <v>2895</v>
@@ -28565,7 +28565,7 @@
         <v>2959</v>
       </c>
       <c r="E267" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F267" t="s">
         <v>2972</v>
@@ -29313,13 +29313,13 @@
         <v>3110</v>
       </c>
       <c r="C279" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D279" t="s">
         <v>1083</v>
       </c>
       <c r="E279" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F279" t="s">
         <v>3098</v>
@@ -29447,7 +29447,7 @@
         <v>2578</v>
       </c>
       <c r="E281" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F281" t="s">
         <v>3098</v>
@@ -29569,7 +29569,7 @@
         <v>3151</v>
       </c>
       <c r="C283" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D283" t="s">
         <v>1353</v>
@@ -29767,7 +29767,7 @@
         <v>2742</v>
       </c>
       <c r="E286" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F286" t="s">
         <v>3177</v>
@@ -29808,13 +29808,13 @@
       <c r="R286"/>
       <c r="S286"/>
       <c r="T286" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U286" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V286" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="287">
@@ -30205,7 +30205,7 @@
         <v>2557</v>
       </c>
       <c r="E293" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="F293" t="s">
         <v>3217</v>
@@ -30331,7 +30331,7 @@
         <v>3262</v>
       </c>
       <c r="E295" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F295" t="s">
         <v>3263</v>
@@ -30451,7 +30451,7 @@
         <v>3281</v>
       </c>
       <c r="C297" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D297" t="s">
         <v>3282</v>
@@ -30515,7 +30515,7 @@
         <v>3291</v>
       </c>
       <c r="C298" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D298" t="s">
         <v>3292</v>
@@ -30707,7 +30707,7 @@
         <v>3324</v>
       </c>
       <c r="C301" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D301" t="s">
         <v>1884</v>
@@ -30777,7 +30777,7 @@
         <v>3334</v>
       </c>
       <c r="E302" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F302" t="s">
         <v>3335</v>
@@ -30901,7 +30901,7 @@
         <v>1564</v>
       </c>
       <c r="E304" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F304" t="s">
         <v>3358</v>
@@ -30942,13 +30942,13 @@
       <c r="R304"/>
       <c r="S304"/>
       <c r="T304" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U304" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V304" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="305">
@@ -30965,7 +30965,7 @@
         <v>1897</v>
       </c>
       <c r="E305" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F305" t="s">
         <v>3367</v>
@@ -31023,7 +31023,7 @@
         <v>3375</v>
       </c>
       <c r="C306" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D306" t="s">
         <v>3376</v>
@@ -31093,7 +31093,7 @@
         <v>3389</v>
       </c>
       <c r="E307" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F307" t="s">
         <v>3390</v>
@@ -31151,7 +31151,7 @@
         <v>3401</v>
       </c>
       <c r="C308" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D308" t="s">
         <v>2804</v>
@@ -31215,13 +31215,13 @@
         <v>3413</v>
       </c>
       <c r="C309" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D309" t="s">
         <v>1628</v>
       </c>
       <c r="E309" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F309" t="s">
         <v>3414</v>
@@ -31349,7 +31349,7 @@
         <v>2695</v>
       </c>
       <c r="E311" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F311" t="s">
         <v>3432</v>
@@ -31477,7 +31477,7 @@
         <v>2578</v>
       </c>
       <c r="E313" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F313" t="s">
         <v>3453</v>
@@ -31539,7 +31539,7 @@
         <v>1564</v>
       </c>
       <c r="E314" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F314" t="s">
         <v>3461</v>
@@ -31723,7 +31723,7 @@
         <v>3493</v>
       </c>
       <c r="C317" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D317" t="s">
         <v>3494</v>
@@ -31793,7 +31793,7 @@
         <v>3504</v>
       </c>
       <c r="E318" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F318" t="s">
         <v>3505</v>
@@ -31851,7 +31851,7 @@
         <v>3513</v>
       </c>
       <c r="C319" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D319" t="s">
         <v>2599</v>
@@ -31985,7 +31985,7 @@
         <v>2742</v>
       </c>
       <c r="E321" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F321" t="s">
         <v>3514</v>
@@ -32113,7 +32113,7 @@
         <v>1409</v>
       </c>
       <c r="E323" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F323" t="s">
         <v>3557</v>
@@ -32154,13 +32154,13 @@
       <c r="R323"/>
       <c r="S323"/>
       <c r="T323" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="U323" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="V323" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
     <row r="324">
@@ -32171,7 +32171,7 @@
         <v>3565</v>
       </c>
       <c r="C324" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D324" t="s">
         <v>3566</v>
@@ -32363,13 +32363,13 @@
         <v>3593</v>
       </c>
       <c r="C327" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D327" t="s">
         <v>2959</v>
       </c>
       <c r="E327" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F327" t="s">
         <v>3594</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-06-04
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -17747,9 +17747,15 @@
         <v>354</v>
       </c>
       <c r="S95"/>
-      <c r="T95"/>
-      <c r="U95"/>
-      <c r="V95"/>
+      <c r="T95" t="s">
+        <v>294</v>
+      </c>
+      <c r="U95" t="s">
+        <v>295</v>
+      </c>
+      <c r="V95" t="s">
+        <v>296</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">

</xml_diff>

<commit_message>
Update parliament data - 2026-06-08
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -179,21 +179,54 @@
     <t xml:space="preserve">Politica nazionale|Media e comunicazione|Protezione sociale</t>
   </si>
   <si>
+    <t xml:space="preserve">26.7321</t>
+  </si>
+  <si>
+    <t xml:space="preserve">de Quattro Jacqueline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EJPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Georgische Staatsangehörige: überdurchschnittlich hohe Gesundheitskosten </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Géorgiens : des coûts médicaux supérieurs à la moyenne </t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Un audit du Contrôle fédéral des finances confirme des coûts médicaux très supérieurs à la moyenne pour les requérants géorgiens, soit 44,40&amp;nbsp;fr par jour et par personne. Entre 2022 et 2025, 26 d’entre eux ont été pris en charge par le SEM pour des traitements lourds. Parmi eux, 17 cas ont bénéficié d’un soutien financier total ou partiel du SEM pour 2,5&amp;nbsp;millions. Avec un cas allant jusqu’à 1,37&amp;nbsp;million. Quand et comment le Conseil fédéral va-t-il enrayer ce tourisme médical ?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Eine Prüfung der Eidgenössischen Finanzkontrolle zeigt, dass die medizinischen Kosten für georgische Asylsuchende mit Fr.&amp;nbsp;44.40 pro Tag und Person deutlich über dem Durchschnitt liegen. Zwischen 2022 und 2025 benötigten 26&amp;nbsp;Asylsuchende Kostengutsprachen des Staatssekretariats für Migration&amp;nbsp;(SEM) für aufwändige Behandlungen. 17 von ihnen erhielten eine vollständige oder teilweise finanzielle Unterstützung durch das SEM im Gesamtumfang von 2,5&amp;nbsp;Millionen&amp;nbsp;Franken. In einem Fall lagen die Kosten bei bis zu 1,37&amp;nbsp;Millionen&amp;nbsp;Franken. Wann und wie wird der Bundesrat diesem Medizintourismus Einhalt gebieten?&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267321</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267321</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Élu &amp; Conseil fédéral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finanzwesen|Migration|Gesundheit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finances|Politique migratoire|Santé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finanze|Migrazione|Salute</t>
+  </si>
+  <si>
     <t xml:space="preserve">26.7324</t>
   </si>
   <si>
-    <t xml:space="preserve">de Quattro Jacqueline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PLR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EJPD</t>
-  </si>
-  <si>
     <t xml:space="preserve">Schwachstellen im Staatssekretariat für Migration </t>
   </si>
   <si>
@@ -267,39 +300,6 @@
   </si>
   <si>
     <t xml:space="preserve">Politica nazionale|Finanze|Media e comunicazione</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.7321</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Georgische Staatsangehörige: überdurchschnittlich hohe Gesundheitskosten </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Géorgiens : des coûts médicaux supérieurs à la moyenne </t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Un audit du Contrôle fédéral des finances confirme des coûts médicaux très supérieurs à la moyenne pour les requérants géorgiens, soit 44,40&amp;nbsp;fr par jour et par personne. Entre 2022 et 2025, 26 d’entre eux ont été pris en charge par le SEM pour des traitements lourds. Parmi eux, 17 cas ont bénéficié d’un soutien financier total ou partiel du SEM pour 2,5&amp;nbsp;millions. Avec un cas allant jusqu’à 1,37&amp;nbsp;million. Quand et comment le Conseil fédéral va-t-il enrayer ce tourisme médical ?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;p&gt;Eine Prüfung der Eidgenössischen Finanzkontrolle zeigt, dass die medizinischen Kosten für georgische Asylsuchende mit Fr.&amp;nbsp;44.40 pro Tag und Person deutlich über dem Durchschnitt liegen. Zwischen 2022 und 2025 benötigten 26&amp;nbsp;Asylsuchende Kostengutsprachen des Staatssekretariats für Migration&amp;nbsp;(SEM) für aufwändige Behandlungen. 17 von ihnen erhielten eine vollständige oder teilweise finanzielle Unterstützung durch das SEM im Gesamtumfang von 2,5&amp;nbsp;Millionen&amp;nbsp;Franken. In einem Fall lagen die Kosten bei bis zu 1,37&amp;nbsp;Millionen&amp;nbsp;Franken. Wann und wie wird der Bundesrat diesem Medizintourismus Einhalt gebieten?&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267321</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267321</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Élu &amp; Conseil fédéral</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finanzwesen|Migration|Gesundheit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finances|Politique migratoire|Santé</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finanze|Migrazione|Salute</t>
   </si>
   <si>
     <t xml:space="preserve">26.3335</t>
@@ -11838,7 +11838,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>20267324</v>
+        <v>20267321</v>
       </c>
       <c r="B4" t="s">
         <v>55</v>
@@ -11884,124 +11884,124 @@
         <v>65</v>
       </c>
       <c r="Q4" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="R4" t="s">
         <v>37</v>
       </c>
       <c r="S4"/>
       <c r="T4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="U4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="V4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>20263550</v>
+        <v>20267324</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C5" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" t="s">
+        <v>57</v>
+      </c>
+      <c r="F5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" t="s">
+        <v>59</v>
+      </c>
+      <c r="I5" t="s">
         <v>71</v>
       </c>
-      <c r="E5" t="s">
+      <c r="J5" t="s">
         <v>72</v>
       </c>
-      <c r="F5" t="s">
-        <v>44</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="K5"/>
+      <c r="L5" t="s">
         <v>73</v>
       </c>
-      <c r="H5"/>
-      <c r="I5" t="s">
+      <c r="M5" t="s">
         <v>74</v>
       </c>
-      <c r="J5" t="s">
+      <c r="N5" t="s">
+        <v>33</v>
+      </c>
+      <c r="O5" t="s">
         <v>75</v>
       </c>
-      <c r="K5" t="s">
+      <c r="P5" t="s">
         <v>76</v>
       </c>
-      <c r="L5"/>
-      <c r="M5" t="s">
-        <v>77</v>
-      </c>
-      <c r="N5" t="s">
-        <v>78</v>
-      </c>
-      <c r="O5" t="s">
-        <v>79</v>
-      </c>
-      <c r="P5" t="s">
-        <v>80</v>
-      </c>
       <c r="Q5" t="s">
-        <v>81</v>
+        <v>36</v>
       </c>
       <c r="R5" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="S5"/>
       <c r="T5" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="U5" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="V5" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>20267321</v>
+        <v>20263550</v>
       </c>
       <c r="B6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" t="s">
+        <v>82</v>
+      </c>
+      <c r="E6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G6" t="s">
+        <v>84</v>
+      </c>
+      <c r="H6"/>
+      <c r="I6" t="s">
         <v>85</v>
       </c>
-      <c r="C6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" t="s">
-        <v>56</v>
-      </c>
-      <c r="E6" t="s">
-        <v>57</v>
-      </c>
-      <c r="F6" t="s">
-        <v>58</v>
-      </c>
-      <c r="G6" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" t="s">
-        <v>59</v>
-      </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>86</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>87</v>
       </c>
-      <c r="K6"/>
-      <c r="L6" t="s">
+      <c r="L6"/>
+      <c r="M6" t="s">
         <v>88</v>
       </c>
-      <c r="M6" t="s">
+      <c r="N6" t="s">
         <v>89</v>
-      </c>
-      <c r="N6" t="s">
-        <v>33</v>
       </c>
       <c r="O6" t="s">
         <v>90</v>
@@ -12013,11 +12013,9 @@
         <v>92</v>
       </c>
       <c r="R6" t="s">
-        <v>37</v>
-      </c>
-      <c r="S6" t="s">
-        <v>37</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="S6"/>
       <c r="T6" t="s">
         <v>93</v>
       </c>
@@ -12036,7 +12034,7 @@
         <v>96</v>
       </c>
       <c r="C7" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D7" t="s">
         <v>97</v>
@@ -12180,7 +12178,7 @@
         <v>99</v>
       </c>
       <c r="G9" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H9" t="s">
         <v>45</v>
@@ -12246,7 +12244,7 @@
         <v>99</v>
       </c>
       <c r="G10" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H10" t="s">
         <v>145</v>
@@ -12300,19 +12298,19 @@
         <v>153</v>
       </c>
       <c r="C11" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D11" t="s">
         <v>154</v>
       </c>
       <c r="E11" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F11" t="s">
         <v>155</v>
       </c>
       <c r="G11" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H11" t="s">
         <v>156</v>
@@ -12408,7 +12406,7 @@
         <v>177</v>
       </c>
       <c r="Q12" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R12" t="s">
         <v>178</v>
@@ -12438,7 +12436,7 @@
         <v>183</v>
       </c>
       <c r="E13" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F13" t="s">
         <v>170</v>
@@ -12474,7 +12472,7 @@
         <v>190</v>
       </c>
       <c r="Q13" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R13" t="s">
         <v>178</v>
@@ -12498,7 +12496,7 @@
         <v>194</v>
       </c>
       <c r="C14" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D14" t="s">
         <v>195</v>
@@ -12540,7 +12538,7 @@
         <v>202</v>
       </c>
       <c r="Q14" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R14" t="s">
         <v>178</v>
@@ -12564,13 +12562,13 @@
         <v>206</v>
       </c>
       <c r="C15" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D15" t="s">
         <v>207</v>
       </c>
       <c r="E15" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F15" t="s">
         <v>155</v>
@@ -12630,7 +12628,7 @@
         <v>218</v>
       </c>
       <c r="C16" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D16" t="s">
         <v>219</v>
@@ -12696,7 +12694,7 @@
         <v>231</v>
       </c>
       <c r="C17" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D17" t="s">
         <v>232</v>
@@ -12762,7 +12760,7 @@
         <v>245</v>
       </c>
       <c r="C18" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D18" t="s">
         <v>246</v>
@@ -12804,7 +12802,7 @@
         <v>254</v>
       </c>
       <c r="Q18" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R18" t="s">
         <v>241</v>
@@ -12870,7 +12868,7 @@
         <v>266</v>
       </c>
       <c r="Q19" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R19" t="s">
         <v>170</v>
@@ -12894,7 +12892,7 @@
         <v>270</v>
       </c>
       <c r="C20" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D20" t="s">
         <v>271</v>
@@ -12936,7 +12934,7 @@
         <v>279</v>
       </c>
       <c r="Q20" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R20" t="s">
         <v>170</v>
@@ -12960,7 +12958,7 @@
         <v>283</v>
       </c>
       <c r="C21" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D21" t="s">
         <v>284</v>
@@ -13026,7 +13024,7 @@
         <v>296</v>
       </c>
       <c r="C22" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D22" t="s">
         <v>297</v>
@@ -13092,7 +13090,7 @@
         <v>308</v>
       </c>
       <c r="C23" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D23" t="s">
         <v>309</v>
@@ -13104,7 +13102,7 @@
         <v>285</v>
       </c>
       <c r="G23" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H23" t="s">
         <v>233</v>
@@ -13262,7 +13260,7 @@
         <v>341</v>
       </c>
       <c r="Q25" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R25" t="s">
         <v>342</v>
@@ -13326,7 +13324,7 @@
         <v>351</v>
       </c>
       <c r="Q26" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R26" t="s">
         <v>342</v>
@@ -13390,7 +13388,7 @@
         <v>363</v>
       </c>
       <c r="Q27" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R27" t="s">
         <v>357</v>
@@ -13420,7 +13418,7 @@
         <v>368</v>
       </c>
       <c r="E28" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F28" t="s">
         <v>369</v>
@@ -13486,7 +13484,7 @@
         <v>380</v>
       </c>
       <c r="E29" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F29" t="s">
         <v>381</v>
@@ -13522,7 +13520,7 @@
         <v>389</v>
       </c>
       <c r="Q29" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R29" t="s">
         <v>390</v>
@@ -13588,7 +13586,7 @@
         <v>403</v>
       </c>
       <c r="Q30" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R30" t="s">
         <v>390</v>
@@ -13612,7 +13610,7 @@
         <v>407</v>
       </c>
       <c r="C31" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D31" t="s">
         <v>24</v>
@@ -13654,7 +13652,7 @@
         <v>414</v>
       </c>
       <c r="Q31" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R31" t="s">
         <v>390</v>
@@ -13690,7 +13688,7 @@
         <v>381</v>
       </c>
       <c r="G32" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H32" t="s">
         <v>247</v>
@@ -13720,7 +13718,7 @@
         <v>423</v>
       </c>
       <c r="Q32" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R32" t="s">
         <v>390</v>
@@ -13744,13 +13742,13 @@
         <v>424</v>
       </c>
       <c r="C33" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D33" t="s">
         <v>425</v>
       </c>
       <c r="E33" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F33" t="s">
         <v>381</v>
@@ -13786,7 +13784,7 @@
         <v>432</v>
       </c>
       <c r="Q33" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R33" t="s">
         <v>390</v>
@@ -13810,7 +13808,7 @@
         <v>436</v>
       </c>
       <c r="C34" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D34" t="s">
         <v>437</v>
@@ -13852,7 +13850,7 @@
         <v>445</v>
       </c>
       <c r="Q34" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R34" t="s">
         <v>390</v>
@@ -13918,7 +13916,7 @@
         <v>456</v>
       </c>
       <c r="Q35" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R35" t="s">
         <v>390</v>
@@ -14008,7 +14006,7 @@
         <v>473</v>
       </c>
       <c r="C37" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D37" t="s">
         <v>474</v>
@@ -14020,7 +14018,7 @@
         <v>475</v>
       </c>
       <c r="G37" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H37" t="s">
         <v>247</v>
@@ -14050,7 +14048,7 @@
         <v>482</v>
       </c>
       <c r="Q37" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R37" t="s">
         <v>390</v>
@@ -14086,7 +14084,7 @@
         <v>475</v>
       </c>
       <c r="G38" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H38" t="s">
         <v>233</v>
@@ -14146,7 +14144,7 @@
         <v>499</v>
       </c>
       <c r="E39" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F39" t="s">
         <v>500</v>
@@ -14210,7 +14208,7 @@
         <v>511</v>
       </c>
       <c r="E40" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F40" t="s">
         <v>500</v>
@@ -14228,7 +14226,7 @@
         <v>513</v>
       </c>
       <c r="K40" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="L40" t="s">
         <v>514</v>
@@ -14270,7 +14268,7 @@
         <v>521</v>
       </c>
       <c r="C41" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D41" t="s">
         <v>522</v>
@@ -14312,7 +14310,7 @@
         <v>531</v>
       </c>
       <c r="Q41" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R41" t="s">
         <v>390</v>
@@ -14378,7 +14376,7 @@
         <v>544</v>
       </c>
       <c r="Q42" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R42" t="s">
         <v>390</v>
@@ -14444,7 +14442,7 @@
         <v>557</v>
       </c>
       <c r="Q43" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R43" t="s">
         <v>390</v>
@@ -14468,7 +14466,7 @@
         <v>561</v>
       </c>
       <c r="C44" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D44" t="s">
         <v>562</v>
@@ -14510,7 +14508,7 @@
         <v>569</v>
       </c>
       <c r="Q44" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R44" t="s">
         <v>390</v>
@@ -14606,7 +14604,7 @@
         <v>586</v>
       </c>
       <c r="E46" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F46" t="s">
         <v>550</v>
@@ -14678,7 +14676,7 @@
         <v>599</v>
       </c>
       <c r="G47" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H47" t="s">
         <v>145</v>
@@ -14732,7 +14730,7 @@
         <v>610</v>
       </c>
       <c r="C48" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D48" t="s">
         <v>611</v>
@@ -14744,7 +14742,7 @@
         <v>599</v>
       </c>
       <c r="G48" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H48" t="s">
         <v>59</v>
@@ -14798,7 +14796,7 @@
         <v>622</v>
       </c>
       <c r="C49" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D49" t="s">
         <v>623</v>
@@ -14840,7 +14838,7 @@
         <v>630</v>
       </c>
       <c r="Q49" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R49" t="s">
         <v>390</v>
@@ -14864,7 +14862,7 @@
         <v>634</v>
       </c>
       <c r="C50" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D50" t="s">
         <v>143</v>
@@ -14876,7 +14874,7 @@
         <v>599</v>
       </c>
       <c r="G50" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H50" t="s">
         <v>59</v>
@@ -14930,7 +14928,7 @@
         <v>645</v>
       </c>
       <c r="C51" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D51" t="s">
         <v>623</v>
@@ -14996,7 +14994,7 @@
         <v>653</v>
       </c>
       <c r="C52" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D52" t="s">
         <v>654</v>
@@ -15038,7 +15036,7 @@
         <v>662</v>
       </c>
       <c r="Q52" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R52" t="s">
         <v>390</v>
@@ -15102,7 +15100,7 @@
         <v>673</v>
       </c>
       <c r="Q53" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R53" t="s">
         <v>390</v>
@@ -15296,7 +15294,7 @@
         <v>706</v>
       </c>
       <c r="Q56" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R56" t="s">
         <v>390</v>
@@ -15384,7 +15382,7 @@
         <v>718</v>
       </c>
       <c r="C58" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D58" t="s">
         <v>719</v>
@@ -15456,7 +15454,7 @@
         <v>733</v>
       </c>
       <c r="E59" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F59" t="s">
         <v>721</v>
@@ -15490,7 +15488,7 @@
         <v>739</v>
       </c>
       <c r="Q59" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R59" t="s">
         <v>390</v>
@@ -15578,7 +15576,7 @@
         <v>753</v>
       </c>
       <c r="C61" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D61" t="s">
         <v>754</v>
@@ -15644,7 +15642,7 @@
         <v>766</v>
       </c>
       <c r="C62" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D62" t="s">
         <v>474</v>
@@ -15656,7 +15654,7 @@
         <v>755</v>
       </c>
       <c r="G62" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H62" t="s">
         <v>59</v>
@@ -15750,7 +15748,7 @@
         <v>785</v>
       </c>
       <c r="Q63" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R63" t="s">
         <v>390</v>
@@ -15774,7 +15772,7 @@
         <v>789</v>
       </c>
       <c r="C64" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D64" t="s">
         <v>790</v>
@@ -15840,7 +15838,7 @@
         <v>802</v>
       </c>
       <c r="C65" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D65" t="s">
         <v>803</v>
@@ -15882,7 +15880,7 @@
         <v>811</v>
       </c>
       <c r="Q65" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R65" t="s">
         <v>390</v>
@@ -15906,13 +15904,13 @@
         <v>815</v>
       </c>
       <c r="C66" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D66" t="s">
         <v>586</v>
       </c>
       <c r="E66" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F66" t="s">
         <v>816</v>
@@ -15972,7 +15970,7 @@
         <v>827</v>
       </c>
       <c r="C67" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D67" t="s">
         <v>828</v>
@@ -16014,7 +16012,7 @@
         <v>835</v>
       </c>
       <c r="Q67" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R67" t="s">
         <v>390</v>
@@ -16038,7 +16036,7 @@
         <v>836</v>
       </c>
       <c r="C68" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D68" t="s">
         <v>837</v>
@@ -16146,7 +16144,7 @@
         <v>852</v>
       </c>
       <c r="Q69" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R69" t="s">
         <v>390</v>
@@ -16212,7 +16210,7 @@
         <v>863</v>
       </c>
       <c r="Q70" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R70" t="s">
         <v>390</v>
@@ -16236,7 +16234,7 @@
         <v>864</v>
       </c>
       <c r="C71" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D71" t="s">
         <v>865</v>
@@ -16278,7 +16276,7 @@
         <v>872</v>
       </c>
       <c r="Q71" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R71" t="s">
         <v>390</v>
@@ -16302,7 +16300,7 @@
         <v>876</v>
       </c>
       <c r="C72" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D72" t="s">
         <v>877</v>
@@ -16314,7 +16312,7 @@
         <v>878</v>
       </c>
       <c r="G72" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H72" t="s">
         <v>28</v>
@@ -16408,7 +16406,7 @@
         <v>893</v>
       </c>
       <c r="Q73" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R73" t="s">
         <v>390</v>
@@ -16438,7 +16436,7 @@
         <v>586</v>
       </c>
       <c r="E74" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F74" t="s">
         <v>887</v>
@@ -16536,7 +16534,7 @@
         <v>915</v>
       </c>
       <c r="Q75" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R75" t="s">
         <v>390</v>
@@ -16600,7 +16598,7 @@
         <v>925</v>
       </c>
       <c r="Q76" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R76" t="s">
         <v>390</v>
@@ -16624,13 +16622,13 @@
         <v>929</v>
       </c>
       <c r="C77" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D77" t="s">
         <v>930</v>
       </c>
       <c r="E77" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F77" t="s">
         <v>931</v>
@@ -16818,7 +16816,7 @@
         <v>955</v>
       </c>
       <c r="C80" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D80" t="s">
         <v>956</v>
@@ -16860,7 +16858,7 @@
         <v>964</v>
       </c>
       <c r="Q80" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R80" t="s">
         <v>390</v>
@@ -16884,7 +16882,7 @@
         <v>965</v>
       </c>
       <c r="C81" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D81" t="s">
         <v>966</v>
@@ -16992,7 +16990,7 @@
         <v>984</v>
       </c>
       <c r="Q82" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R82" t="s">
         <v>390</v>
@@ -17016,7 +17014,7 @@
         <v>988</v>
       </c>
       <c r="C83" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D83" t="s">
         <v>487</v>
@@ -17028,7 +17026,7 @@
         <v>989</v>
       </c>
       <c r="G83" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H83" t="s">
         <v>233</v>
@@ -17058,7 +17056,7 @@
         <v>996</v>
       </c>
       <c r="Q83" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R83" t="s">
         <v>390</v>
@@ -17082,7 +17080,7 @@
         <v>997</v>
       </c>
       <c r="C84" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D84" t="s">
         <v>998</v>
@@ -17188,7 +17186,7 @@
         <v>1016</v>
       </c>
       <c r="Q85" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R85" t="s">
         <v>390</v>
@@ -17276,7 +17274,7 @@
         <v>1028</v>
       </c>
       <c r="C87" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D87" t="s">
         <v>168</v>
@@ -17318,7 +17316,7 @@
         <v>1036</v>
       </c>
       <c r="Q87" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R87" t="s">
         <v>390</v>
@@ -17348,7 +17346,7 @@
         <v>586</v>
       </c>
       <c r="E88" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F88" t="s">
         <v>1041</v>
@@ -17408,7 +17406,7 @@
         <v>1049</v>
       </c>
       <c r="C89" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D89" t="s">
         <v>297</v>
@@ -17480,7 +17478,7 @@
         <v>1061</v>
       </c>
       <c r="E90" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F90" t="s">
         <v>1062</v>
@@ -17580,7 +17578,7 @@
         <v>1078</v>
       </c>
       <c r="Q91" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R91" t="s">
         <v>390</v>
@@ -17644,7 +17642,7 @@
         <v>1089</v>
       </c>
       <c r="Q92" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R92" t="s">
         <v>390</v>
@@ -17668,7 +17666,7 @@
         <v>1090</v>
       </c>
       <c r="C93" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D93" t="s">
         <v>24</v>
@@ -17710,7 +17708,7 @@
         <v>1098</v>
       </c>
       <c r="Q93" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R93" t="s">
         <v>390</v>
@@ -17734,7 +17732,7 @@
         <v>1102</v>
       </c>
       <c r="C94" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D94" t="s">
         <v>1103</v>
@@ -17800,13 +17798,13 @@
         <v>1115</v>
       </c>
       <c r="C95" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D95" t="s">
         <v>1116</v>
       </c>
       <c r="E95" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F95" t="s">
         <v>1117</v>
@@ -17842,7 +17840,7 @@
         <v>1124</v>
       </c>
       <c r="Q95" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R95" t="s">
         <v>390</v>
@@ -17866,13 +17864,13 @@
         <v>1128</v>
       </c>
       <c r="C96" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D96" t="s">
         <v>1129</v>
       </c>
       <c r="E96" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F96" t="s">
         <v>1130</v>
@@ -17942,7 +17940,7 @@
         <v>1143</v>
       </c>
       <c r="G97" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H97" t="s">
         <v>59</v>
@@ -17972,7 +17970,7 @@
         <v>1150</v>
       </c>
       <c r="Q97" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R97" t="s">
         <v>390</v>
@@ -17996,13 +17994,13 @@
         <v>1154</v>
       </c>
       <c r="C98" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D98" t="s">
         <v>207</v>
       </c>
       <c r="E98" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F98" t="s">
         <v>1155</v>
@@ -18038,7 +18036,7 @@
         <v>1162</v>
       </c>
       <c r="Q98" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R98" t="s">
         <v>390</v>
@@ -18102,7 +18100,7 @@
         <v>1170</v>
       </c>
       <c r="Q99" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R99" t="s">
         <v>390</v>
@@ -18132,7 +18130,7 @@
         <v>733</v>
       </c>
       <c r="E100" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F100" t="s">
         <v>1175</v>
@@ -18168,7 +18166,7 @@
         <v>1182</v>
       </c>
       <c r="Q100" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R100" t="s">
         <v>390</v>
@@ -18192,7 +18190,7 @@
         <v>1183</v>
       </c>
       <c r="C101" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D101" t="s">
         <v>461</v>
@@ -18234,7 +18232,7 @@
         <v>1190</v>
       </c>
       <c r="Q101" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R101" t="s">
         <v>390</v>
@@ -18258,7 +18256,7 @@
         <v>1191</v>
       </c>
       <c r="C102" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D102" t="s">
         <v>1192</v>
@@ -18300,7 +18298,7 @@
         <v>1200</v>
       </c>
       <c r="Q102" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R102" t="s">
         <v>390</v>
@@ -18366,7 +18364,7 @@
         <v>1213</v>
       </c>
       <c r="Q103" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R103" t="s">
         <v>390</v>
@@ -18393,16 +18391,16 @@
         <v>113</v>
       </c>
       <c r="D104" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="E104" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F104" t="s">
         <v>1206</v>
       </c>
       <c r="G104" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H104" t="s">
         <v>115</v>
@@ -18432,7 +18430,7 @@
         <v>1224</v>
       </c>
       <c r="Q104" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R104" t="s">
         <v>390</v>
@@ -18498,7 +18496,7 @@
         <v>1236</v>
       </c>
       <c r="Q105" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R105" t="s">
         <v>390</v>
@@ -18564,7 +18562,7 @@
         <v>1245</v>
       </c>
       <c r="Q106" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R106" t="s">
         <v>390</v>
@@ -18588,7 +18586,7 @@
         <v>1249</v>
       </c>
       <c r="C107" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D107" t="s">
         <v>837</v>
@@ -18630,7 +18628,7 @@
         <v>1256</v>
       </c>
       <c r="Q107" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R107" t="s">
         <v>390</v>
@@ -18720,7 +18718,7 @@
         <v>1272</v>
       </c>
       <c r="C109" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D109" t="s">
         <v>1273</v>
@@ -18786,7 +18784,7 @@
         <v>1285</v>
       </c>
       <c r="C110" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D110" t="s">
         <v>195</v>
@@ -18828,7 +18826,7 @@
         <v>1293</v>
       </c>
       <c r="Q110" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R110" t="s">
         <v>390</v>
@@ -18852,7 +18850,7 @@
         <v>1297</v>
       </c>
       <c r="C111" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D111" t="s">
         <v>1298</v>
@@ -18894,7 +18892,7 @@
         <v>1305</v>
       </c>
       <c r="Q111" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R111" t="s">
         <v>390</v>
@@ -18918,7 +18916,7 @@
         <v>1309</v>
       </c>
       <c r="C112" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D112" t="s">
         <v>908</v>
@@ -18960,7 +18958,7 @@
         <v>1316</v>
       </c>
       <c r="Q112" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R112" t="s">
         <v>390</v>
@@ -18984,7 +18982,7 @@
         <v>1317</v>
       </c>
       <c r="C113" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D113" t="s">
         <v>1318</v>
@@ -19092,7 +19090,7 @@
         <v>1335</v>
       </c>
       <c r="Q114" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R114" t="s">
         <v>390</v>
@@ -19158,7 +19156,7 @@
         <v>1347</v>
       </c>
       <c r="Q115" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R115" t="s">
         <v>390</v>
@@ -19224,7 +19222,7 @@
         <v>1358</v>
       </c>
       <c r="Q116" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R116" t="s">
         <v>390</v>
@@ -19290,20 +19288,20 @@
         <v>1371</v>
       </c>
       <c r="Q117" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R117" t="s">
         <v>390</v>
       </c>
       <c r="S117"/>
       <c r="T117" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="U117" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="V117" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="118">
@@ -19314,7 +19312,7 @@
         <v>1372</v>
       </c>
       <c r="C118" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D118" t="s">
         <v>966</v>
@@ -19386,7 +19384,7 @@
         <v>586</v>
       </c>
       <c r="E119" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F119" t="s">
         <v>1364</v>
@@ -19446,7 +19444,7 @@
         <v>1391</v>
       </c>
       <c r="C120" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D120" t="s">
         <v>1392</v>
@@ -19578,7 +19576,7 @@
         <v>1415</v>
       </c>
       <c r="C122" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D122" t="s">
         <v>1103</v>
@@ -19644,7 +19642,7 @@
         <v>1423</v>
       </c>
       <c r="C123" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D123" t="s">
         <v>711</v>
@@ -19686,7 +19684,7 @@
         <v>1431</v>
       </c>
       <c r="Q123" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R123" t="s">
         <v>390</v>
@@ -19716,7 +19714,7 @@
         <v>1433</v>
       </c>
       <c r="E124" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F124" t="s">
         <v>1424</v>
@@ -19752,7 +19750,7 @@
         <v>1440</v>
       </c>
       <c r="Q124" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R124" t="s">
         <v>390</v>
@@ -19816,7 +19814,7 @@
         <v>1448</v>
       </c>
       <c r="Q125" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R125" t="s">
         <v>390</v>
@@ -19880,7 +19878,7 @@
         <v>1458</v>
       </c>
       <c r="Q126" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R126" t="s">
         <v>390</v>
@@ -19904,7 +19902,7 @@
         <v>1462</v>
       </c>
       <c r="C127" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D127" t="s">
         <v>1463</v>
@@ -19946,7 +19944,7 @@
         <v>1471</v>
       </c>
       <c r="Q127" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R127" t="s">
         <v>390</v>
@@ -19970,7 +19968,7 @@
         <v>1475</v>
       </c>
       <c r="C128" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D128" t="s">
         <v>908</v>
@@ -20012,7 +20010,7 @@
         <v>1482</v>
       </c>
       <c r="Q128" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R128" t="s">
         <v>390</v>
@@ -20036,7 +20034,7 @@
         <v>1483</v>
       </c>
       <c r="C129" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D129" t="s">
         <v>1484</v>
@@ -20102,7 +20100,7 @@
         <v>1493</v>
       </c>
       <c r="C130" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D130" t="s">
         <v>143</v>
@@ -20174,7 +20172,7 @@
         <v>1506</v>
       </c>
       <c r="E131" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F131" t="s">
         <v>1507</v>
@@ -20338,7 +20336,7 @@
         <v>1535</v>
       </c>
       <c r="Q133" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R133" t="s">
         <v>390</v>
@@ -20368,7 +20366,7 @@
         <v>1540</v>
       </c>
       <c r="E134" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F134" t="s">
         <v>1541</v>
@@ -20402,7 +20400,7 @@
         <v>1547</v>
       </c>
       <c r="Q134" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R134" t="s">
         <v>390</v>
@@ -20468,7 +20466,7 @@
         <v>1557</v>
       </c>
       <c r="Q135" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R135" t="s">
         <v>390</v>
@@ -20492,7 +20490,7 @@
         <v>1561</v>
       </c>
       <c r="C136" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D136" t="s">
         <v>865</v>
@@ -20558,7 +20556,7 @@
         <v>1573</v>
       </c>
       <c r="C137" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D137" t="s">
         <v>1574</v>
@@ -20598,7 +20596,7 @@
         <v>1582</v>
       </c>
       <c r="Q137" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R137" t="s">
         <v>390</v>
@@ -20662,7 +20660,7 @@
         <v>1593</v>
       </c>
       <c r="Q138" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R138" t="s">
         <v>390</v>
@@ -20686,7 +20684,7 @@
         <v>1597</v>
       </c>
       <c r="C139" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D139" t="s">
         <v>56</v>
@@ -20728,7 +20726,7 @@
         <v>1605</v>
       </c>
       <c r="Q139" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R139" t="s">
         <v>390</v>
@@ -20752,13 +20750,13 @@
         <v>1609</v>
       </c>
       <c r="C140" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D140" t="s">
         <v>1610</v>
       </c>
       <c r="E140" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F140" t="s">
         <v>1611</v>
@@ -20882,7 +20880,7 @@
         <v>1633</v>
       </c>
       <c r="C142" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D142" t="s">
         <v>1634</v>
@@ -20894,7 +20892,7 @@
         <v>1635</v>
       </c>
       <c r="G142" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H142" t="s">
         <v>59</v>
@@ -20990,7 +20988,7 @@
         <v>1655</v>
       </c>
       <c r="Q143" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R143" t="s">
         <v>390</v>
@@ -21014,7 +21012,7 @@
         <v>1659</v>
       </c>
       <c r="C144" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D144" t="s">
         <v>711</v>
@@ -21056,7 +21054,7 @@
         <v>1666</v>
       </c>
       <c r="Q144" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R144" t="s">
         <v>390</v>
@@ -21080,7 +21078,7 @@
         <v>1667</v>
       </c>
       <c r="C145" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D145" t="s">
         <v>1668</v>
@@ -21122,7 +21120,7 @@
         <v>1675</v>
       </c>
       <c r="Q145" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R145" t="s">
         <v>390</v>
@@ -21218,7 +21216,7 @@
         <v>1693</v>
       </c>
       <c r="E147" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F147" t="s">
         <v>1681</v>
@@ -21316,7 +21314,7 @@
         <v>1710</v>
       </c>
       <c r="Q148" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R148" t="s">
         <v>390</v>
@@ -21404,7 +21402,7 @@
         <v>1721</v>
       </c>
       <c r="C150" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D150" t="s">
         <v>711</v>
@@ -21446,7 +21444,7 @@
         <v>1729</v>
       </c>
       <c r="Q150" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R150" t="s">
         <v>390</v>
@@ -21512,7 +21510,7 @@
         <v>1741</v>
       </c>
       <c r="Q151" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R151" t="s">
         <v>390</v>
@@ -21542,7 +21540,7 @@
         <v>1610</v>
       </c>
       <c r="E152" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F152" t="s">
         <v>1734</v>
@@ -21602,13 +21600,13 @@
         <v>1756</v>
       </c>
       <c r="C153" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D153" t="s">
         <v>1757</v>
       </c>
       <c r="E153" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F153" t="s">
         <v>1734</v>
@@ -21644,7 +21642,7 @@
         <v>1764</v>
       </c>
       <c r="Q153" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R153" t="s">
         <v>390</v>
@@ -21674,13 +21672,13 @@
         <v>154</v>
       </c>
       <c r="E154" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F154" t="s">
         <v>1769</v>
       </c>
       <c r="G154" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H154" t="s">
         <v>247</v>
@@ -21734,7 +21732,7 @@
         <v>1780</v>
       </c>
       <c r="C155" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D155" t="s">
         <v>1392</v>
@@ -21776,7 +21774,7 @@
         <v>1788</v>
       </c>
       <c r="Q155" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R155" t="s">
         <v>390</v>
@@ -21800,13 +21798,13 @@
         <v>1792</v>
       </c>
       <c r="C156" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D156" t="s">
         <v>1433</v>
       </c>
       <c r="E156" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F156" t="s">
         <v>1793</v>
@@ -21842,7 +21840,7 @@
         <v>1800</v>
       </c>
       <c r="Q156" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R156" t="s">
         <v>390</v>
@@ -21866,7 +21864,7 @@
         <v>1801</v>
       </c>
       <c r="C157" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D157" t="s">
         <v>1071</v>
@@ -21908,7 +21906,7 @@
         <v>1809</v>
       </c>
       <c r="Q157" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R157" t="s">
         <v>390</v>
@@ -21972,20 +21970,20 @@
         <v>1818</v>
       </c>
       <c r="Q158" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R158" t="s">
         <v>390</v>
       </c>
       <c r="S158"/>
       <c r="T158" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="U158" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="V158" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="159">
@@ -22036,20 +22034,20 @@
         <v>1825</v>
       </c>
       <c r="Q159" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R159" t="s">
         <v>390</v>
       </c>
       <c r="S159"/>
       <c r="T159" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="U159" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="V159" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="160">
@@ -22060,7 +22058,7 @@
         <v>1826</v>
       </c>
       <c r="C160" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D160" t="s">
         <v>1528</v>
@@ -22102,7 +22100,7 @@
         <v>1834</v>
       </c>
       <c r="Q160" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R160" t="s">
         <v>390</v>
@@ -22168,7 +22166,7 @@
         <v>1843</v>
       </c>
       <c r="Q161" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R161" t="s">
         <v>390</v>
@@ -22234,7 +22232,7 @@
         <v>1854</v>
       </c>
       <c r="Q162" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R162" t="s">
         <v>390</v>
@@ -22258,7 +22256,7 @@
         <v>1858</v>
       </c>
       <c r="C163" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D163" t="s">
         <v>1859</v>
@@ -22300,7 +22298,7 @@
         <v>1866</v>
       </c>
       <c r="Q163" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R163" t="s">
         <v>390</v>
@@ -22324,7 +22322,7 @@
         <v>1867</v>
       </c>
       <c r="C164" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D164" t="s">
         <v>1363</v>
@@ -22366,7 +22364,7 @@
         <v>1875</v>
       </c>
       <c r="Q164" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R164" t="s">
         <v>390</v>
@@ -22390,7 +22388,7 @@
         <v>1879</v>
       </c>
       <c r="C165" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D165" t="s">
         <v>114</v>
@@ -22432,7 +22430,7 @@
         <v>1886</v>
       </c>
       <c r="Q165" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R165" t="s">
         <v>390</v>
@@ -22522,7 +22520,7 @@
         <v>1899</v>
       </c>
       <c r="C167" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D167" t="s">
         <v>97</v>
@@ -22564,7 +22562,7 @@
         <v>1907</v>
       </c>
       <c r="Q167" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R167" t="s">
         <v>390</v>
@@ -22588,7 +22586,7 @@
         <v>1911</v>
       </c>
       <c r="C168" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D168" t="s">
         <v>1574</v>
@@ -22692,7 +22690,7 @@
         <v>1930</v>
       </c>
       <c r="Q169" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R169" t="s">
         <v>390</v>
@@ -22756,7 +22754,7 @@
         <v>1937</v>
       </c>
       <c r="Q170" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R170" t="s">
         <v>390</v>
@@ -22790,7 +22788,7 @@
         <v>1940</v>
       </c>
       <c r="G171" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H171" t="s">
         <v>233</v>
@@ -22820,7 +22818,7 @@
         <v>1948</v>
       </c>
       <c r="Q171" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R171" t="s">
         <v>390</v>
@@ -22884,7 +22882,7 @@
         <v>1957</v>
       </c>
       <c r="Q172" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R172" t="s">
         <v>390</v>
@@ -22908,7 +22906,7 @@
         <v>1961</v>
       </c>
       <c r="C173" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D173" t="s">
         <v>1811</v>
@@ -23082,7 +23080,7 @@
         <v>1994</v>
       </c>
       <c r="Q175" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R175" t="s">
         <v>390</v>
@@ -23182,7 +23180,7 @@
         <v>2009</v>
       </c>
       <c r="G177" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H177" t="s">
         <v>1648</v>
@@ -23212,7 +23210,7 @@
         <v>2016</v>
       </c>
       <c r="Q177" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R177" t="s">
         <v>390</v>
@@ -23236,13 +23234,13 @@
         <v>2020</v>
       </c>
       <c r="C178" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D178" t="s">
         <v>2021</v>
       </c>
       <c r="E178" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F178" t="s">
         <v>2009</v>
@@ -23368,7 +23366,7 @@
         <v>2044</v>
       </c>
       <c r="C180" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D180" t="s">
         <v>1528</v>
@@ -23434,7 +23432,7 @@
         <v>2056</v>
       </c>
       <c r="C181" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D181" t="s">
         <v>966</v>
@@ -23476,7 +23474,7 @@
         <v>2063</v>
       </c>
       <c r="Q181" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R181" t="s">
         <v>390</v>
@@ -23542,20 +23540,20 @@
         <v>2074</v>
       </c>
       <c r="Q182" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R182" t="s">
         <v>390</v>
       </c>
       <c r="S182"/>
       <c r="T182" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="U182" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="V182" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="183">
@@ -23566,7 +23564,7 @@
         <v>2075</v>
       </c>
       <c r="C183" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D183" t="s">
         <v>246</v>
@@ -23608,7 +23606,7 @@
         <v>2083</v>
       </c>
       <c r="Q183" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R183" t="s">
         <v>390</v>
@@ -23632,13 +23630,13 @@
         <v>2084</v>
       </c>
       <c r="C184" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D184" t="s">
         <v>2085</v>
       </c>
       <c r="E184" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F184" t="s">
         <v>2086</v>
@@ -23674,7 +23672,7 @@
         <v>2093</v>
       </c>
       <c r="Q184" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R184" t="s">
         <v>390</v>
@@ -23698,7 +23696,7 @@
         <v>2097</v>
       </c>
       <c r="C185" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D185" t="s">
         <v>536</v>
@@ -23806,7 +23804,7 @@
         <v>2117</v>
       </c>
       <c r="Q186" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R186" t="s">
         <v>390</v>
@@ -23830,7 +23828,7 @@
         <v>2118</v>
       </c>
       <c r="C187" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D187" t="s">
         <v>246</v>
@@ -23872,7 +23870,7 @@
         <v>2126</v>
       </c>
       <c r="Q187" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R187" t="s">
         <v>390</v>
@@ -23962,7 +23960,7 @@
         <v>2139</v>
       </c>
       <c r="C189" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D189" t="s">
         <v>2140</v>
@@ -24040,7 +24038,7 @@
         <v>2153</v>
       </c>
       <c r="G190" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H190" t="s">
         <v>1648</v>
@@ -24070,7 +24068,7 @@
         <v>2160</v>
       </c>
       <c r="Q190" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R190" t="s">
         <v>390</v>
@@ -24160,7 +24158,7 @@
         <v>2176</v>
       </c>
       <c r="C192" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D192" t="s">
         <v>2177</v>
@@ -24202,7 +24200,7 @@
         <v>2184</v>
       </c>
       <c r="Q192" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R192" t="s">
         <v>390</v>
@@ -24226,7 +24224,7 @@
         <v>2188</v>
       </c>
       <c r="C193" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D193" t="s">
         <v>1986</v>
@@ -24268,7 +24266,7 @@
         <v>2196</v>
       </c>
       <c r="Q193" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R193" t="s">
         <v>390</v>
@@ -24292,7 +24290,7 @@
         <v>2197</v>
       </c>
       <c r="C194" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D194" t="s">
         <v>2198</v>
@@ -24334,7 +24332,7 @@
         <v>2206</v>
       </c>
       <c r="Q194" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R194" t="s">
         <v>390</v>
@@ -24398,7 +24396,7 @@
         <v>2214</v>
       </c>
       <c r="Q195" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R195" t="s">
         <v>390</v>
@@ -24462,7 +24460,7 @@
         <v>2225</v>
       </c>
       <c r="Q196" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R196" t="s">
         <v>390</v>
@@ -24528,7 +24526,7 @@
         <v>2237</v>
       </c>
       <c r="Q197" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R197" t="s">
         <v>390</v>
@@ -24552,7 +24550,7 @@
         <v>2241</v>
       </c>
       <c r="C198" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D198" t="s">
         <v>2242</v>
@@ -24618,7 +24616,7 @@
         <v>2253</v>
       </c>
       <c r="C199" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D199" t="s">
         <v>2254</v>
@@ -24684,7 +24682,7 @@
         <v>2264</v>
       </c>
       <c r="C200" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D200" t="s">
         <v>1891</v>
@@ -24726,7 +24724,7 @@
         <v>2271</v>
       </c>
       <c r="Q200" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R200" t="s">
         <v>390</v>
@@ -24792,7 +24790,7 @@
         <v>2284</v>
       </c>
       <c r="Q201" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R201" t="s">
         <v>390</v>
@@ -24856,7 +24854,7 @@
         <v>2296</v>
       </c>
       <c r="Q202" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R202" t="s">
         <v>390</v>
@@ -24880,7 +24878,7 @@
         <v>2300</v>
       </c>
       <c r="C203" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D203" t="s">
         <v>908</v>
@@ -24946,13 +24944,13 @@
         <v>2312</v>
       </c>
       <c r="C204" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D204" t="s">
         <v>1757</v>
       </c>
       <c r="E204" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F204" t="s">
         <v>2313</v>
@@ -25076,7 +25074,7 @@
         <v>2333</v>
       </c>
       <c r="C206" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D206" t="s">
         <v>2334</v>
@@ -25142,7 +25140,7 @@
         <v>2346</v>
       </c>
       <c r="C207" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D207" t="s">
         <v>2347</v>
@@ -25278,7 +25276,7 @@
         <v>586</v>
       </c>
       <c r="E209" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F209" t="s">
         <v>2371</v>
@@ -25378,7 +25376,7 @@
         <v>2391</v>
       </c>
       <c r="Q210" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R210" t="s">
         <v>390</v>
@@ -25412,7 +25410,7 @@
         <v>2397</v>
       </c>
       <c r="G211" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H211" t="s">
         <v>145</v>
@@ -25442,7 +25440,7 @@
         <v>2404</v>
       </c>
       <c r="Q211" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R211" t="s">
         <v>390</v>
@@ -25476,7 +25474,7 @@
         <v>2397</v>
       </c>
       <c r="G212" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H212" t="s">
         <v>247</v>
@@ -25506,7 +25504,7 @@
         <v>2415</v>
       </c>
       <c r="Q212" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R212" t="s">
         <v>390</v>
@@ -25536,7 +25534,7 @@
         <v>183</v>
       </c>
       <c r="E213" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F213" t="s">
         <v>369</v>
@@ -25572,7 +25570,7 @@
         <v>2426</v>
       </c>
       <c r="Q213" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R213"/>
       <c r="S213"/>
@@ -25594,7 +25592,7 @@
         <v>2430</v>
       </c>
       <c r="C214" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D214" t="s">
         <v>966</v>
@@ -25670,7 +25668,7 @@
         <v>272</v>
       </c>
       <c r="G215" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H215" t="s">
         <v>233</v>
@@ -25700,7 +25698,7 @@
         <v>2447</v>
       </c>
       <c r="Q215" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R215"/>
       <c r="S215"/>
@@ -25792,7 +25790,7 @@
         <v>2463</v>
       </c>
       <c r="E217" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F217" t="s">
         <v>2464</v>
@@ -25888,7 +25886,7 @@
         <v>2477</v>
       </c>
       <c r="Q218" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R218"/>
       <c r="S218"/>
@@ -25952,7 +25950,7 @@
         <v>2489</v>
       </c>
       <c r="Q219" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R219"/>
       <c r="S219"/>
@@ -26016,7 +26014,7 @@
         <v>2499</v>
       </c>
       <c r="Q220" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R220"/>
       <c r="S220"/>
@@ -26080,7 +26078,7 @@
         <v>2507</v>
       </c>
       <c r="Q221" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R221"/>
       <c r="S221"/>
@@ -26114,7 +26112,7 @@
         <v>2513</v>
       </c>
       <c r="G222" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H222" t="s">
         <v>145</v>
@@ -26178,7 +26176,7 @@
         <v>2513</v>
       </c>
       <c r="G223" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H223" t="s">
         <v>233</v>
@@ -26230,7 +26228,7 @@
         <v>2527</v>
       </c>
       <c r="C224" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D224" t="s">
         <v>1103</v>
@@ -26272,7 +26270,7 @@
         <v>2534</v>
       </c>
       <c r="Q224" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R224"/>
       <c r="S224"/>
@@ -26336,7 +26334,7 @@
         <v>2546</v>
       </c>
       <c r="Q225" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R225"/>
       <c r="S225"/>
@@ -26358,7 +26356,7 @@
         <v>2550</v>
       </c>
       <c r="C226" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D226" t="s">
         <v>2551</v>
@@ -26370,7 +26368,7 @@
         <v>2552</v>
       </c>
       <c r="G226" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H226" t="s">
         <v>233</v>
@@ -26422,7 +26420,7 @@
         <v>2563</v>
       </c>
       <c r="C227" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D227" t="s">
         <v>690</v>
@@ -26464,7 +26462,7 @@
         <v>2571</v>
       </c>
       <c r="Q227" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R227"/>
       <c r="S227"/>
@@ -26588,7 +26586,7 @@
         <v>2585</v>
       </c>
       <c r="Q229" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R229"/>
       <c r="S229"/>
@@ -26650,7 +26648,7 @@
         <v>2595</v>
       </c>
       <c r="Q230" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R230"/>
       <c r="S230"/>
@@ -26740,7 +26738,7 @@
         <v>183</v>
       </c>
       <c r="E232" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F232" t="s">
         <v>322</v>
@@ -26858,7 +26856,7 @@
         <v>2627</v>
       </c>
       <c r="C234" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D234" t="s">
         <v>129</v>
@@ -26870,7 +26868,7 @@
         <v>2628</v>
       </c>
       <c r="G234" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H234" t="s">
         <v>247</v>
@@ -26900,7 +26898,7 @@
         <v>2635</v>
       </c>
       <c r="Q234" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R234"/>
       <c r="S234"/>
@@ -26962,7 +26960,7 @@
         <v>2643</v>
       </c>
       <c r="Q235" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R235"/>
       <c r="S235"/>
@@ -27058,7 +27056,7 @@
         <v>2656</v>
       </c>
       <c r="G237" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H237" t="s">
         <v>145</v>
@@ -27088,7 +27086,7 @@
         <v>2663</v>
       </c>
       <c r="Q237" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R237"/>
       <c r="S237"/>
@@ -27110,13 +27108,13 @@
         <v>2667</v>
       </c>
       <c r="C238" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D238" t="s">
         <v>1433</v>
       </c>
       <c r="E238" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F238" t="s">
         <v>2668</v>
@@ -27152,7 +27150,7 @@
         <v>2675</v>
       </c>
       <c r="Q238" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R238"/>
       <c r="S238"/>
@@ -27174,7 +27172,7 @@
         <v>2679</v>
       </c>
       <c r="C239" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D239" t="s">
         <v>2680</v>
@@ -27216,7 +27214,7 @@
         <v>2688</v>
       </c>
       <c r="Q239" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R239"/>
       <c r="S239"/>
@@ -27278,7 +27276,7 @@
         <v>2699</v>
       </c>
       <c r="Q240" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R240"/>
       <c r="S240"/>
@@ -27300,13 +27298,13 @@
         <v>2700</v>
       </c>
       <c r="C241" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D241" t="s">
         <v>2701</v>
       </c>
       <c r="E241" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F241" t="s">
         <v>2702</v>
@@ -27364,13 +27362,13 @@
         <v>2713</v>
       </c>
       <c r="C242" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D242" t="s">
         <v>183</v>
       </c>
       <c r="E242" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F242" t="s">
         <v>2702</v>
@@ -27406,7 +27404,7 @@
         <v>2720</v>
       </c>
       <c r="Q242" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R242"/>
       <c r="S242"/>
@@ -27428,7 +27426,7 @@
         <v>2721</v>
       </c>
       <c r="C243" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D243" t="s">
         <v>2722</v>
@@ -27498,7 +27496,7 @@
         <v>1757</v>
       </c>
       <c r="E244" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F244" t="s">
         <v>2734</v>
@@ -27556,7 +27554,7 @@
         <v>2742</v>
       </c>
       <c r="C245" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D245" t="s">
         <v>2743</v>
@@ -27598,7 +27596,7 @@
         <v>2750</v>
       </c>
       <c r="Q245" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R245"/>
       <c r="S245"/>
@@ -27620,7 +27618,7 @@
         <v>2751</v>
       </c>
       <c r="C246" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D246" t="s">
         <v>2334</v>
@@ -27684,7 +27682,7 @@
         <v>2763</v>
       </c>
       <c r="C247" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D247" t="s">
         <v>2764</v>
@@ -27696,7 +27694,7 @@
         <v>2752</v>
       </c>
       <c r="G247" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H247" t="s">
         <v>115</v>
@@ -27748,7 +27746,7 @@
         <v>2772</v>
       </c>
       <c r="C248" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D248" t="s">
         <v>334</v>
@@ -27790,7 +27788,7 @@
         <v>2780</v>
       </c>
       <c r="Q248" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R248"/>
       <c r="S248"/>
@@ -27916,7 +27914,7 @@
         <v>2801</v>
       </c>
       <c r="Q250" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R250"/>
       <c r="S250"/>
@@ -27938,7 +27936,7 @@
         <v>2805</v>
       </c>
       <c r="C251" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D251" t="s">
         <v>2782</v>
@@ -28002,13 +28000,13 @@
         <v>2817</v>
       </c>
       <c r="C252" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D252" t="s">
         <v>2818</v>
       </c>
       <c r="E252" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F252" t="s">
         <v>2819</v>
@@ -28044,7 +28042,7 @@
         <v>2826</v>
       </c>
       <c r="Q252" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R252"/>
       <c r="S252"/>
@@ -28072,7 +28070,7 @@
         <v>1433</v>
       </c>
       <c r="E253" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F253" t="s">
         <v>2819</v>
@@ -28108,7 +28106,7 @@
         <v>2837</v>
       </c>
       <c r="Q253" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R253"/>
       <c r="S253"/>
@@ -28130,7 +28128,7 @@
         <v>2841</v>
       </c>
       <c r="C254" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D254" t="s">
         <v>271</v>
@@ -28172,7 +28170,7 @@
         <v>2848</v>
       </c>
       <c r="Q254" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R254"/>
       <c r="S254"/>
@@ -28236,7 +28234,7 @@
         <v>2860</v>
       </c>
       <c r="Q255" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R255"/>
       <c r="S255"/>
@@ -28258,19 +28256,19 @@
         <v>2864</v>
       </c>
       <c r="C256" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D256" t="s">
         <v>2865</v>
       </c>
       <c r="E256" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F256" t="s">
         <v>2853</v>
       </c>
       <c r="G256" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H256" t="s">
         <v>145</v>
@@ -28300,7 +28298,7 @@
         <v>2872</v>
       </c>
       <c r="Q256" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R256"/>
       <c r="S256"/>
@@ -28322,7 +28320,7 @@
         <v>2876</v>
       </c>
       <c r="C257" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D257" t="s">
         <v>2877</v>
@@ -28364,7 +28362,7 @@
         <v>2885</v>
       </c>
       <c r="Q257" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R257"/>
       <c r="S257"/>
@@ -28428,7 +28426,7 @@
         <v>2899</v>
       </c>
       <c r="Q258" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R258"/>
       <c r="S258"/>
@@ -28616,7 +28614,7 @@
         <v>2925</v>
       </c>
       <c r="Q261" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R261"/>
       <c r="S261"/>
@@ -28638,7 +28636,7 @@
         <v>2926</v>
       </c>
       <c r="C262" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D262" t="s">
         <v>2927</v>
@@ -28680,7 +28678,7 @@
         <v>2935</v>
       </c>
       <c r="Q262" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R262"/>
       <c r="S262"/>
@@ -28744,7 +28742,7 @@
         <v>2943</v>
       </c>
       <c r="Q263" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R263"/>
       <c r="S263"/>
@@ -28806,7 +28804,7 @@
         <v>2954</v>
       </c>
       <c r="Q264" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R264"/>
       <c r="S264"/>
@@ -28868,7 +28866,7 @@
         <v>2962</v>
       </c>
       <c r="Q265" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R265"/>
       <c r="S265"/>
@@ -28930,7 +28928,7 @@
         <v>2972</v>
       </c>
       <c r="Q266" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R266"/>
       <c r="S266"/>
@@ -28952,7 +28950,7 @@
         <v>2973</v>
       </c>
       <c r="C267" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D267" t="s">
         <v>1519</v>
@@ -29054,7 +29052,7 @@
         <v>2994</v>
       </c>
       <c r="Q268" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R268"/>
       <c r="S268"/>
@@ -29088,7 +29086,7 @@
         <v>3000</v>
       </c>
       <c r="G269" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H269" t="s">
         <v>45</v>
@@ -29118,7 +29116,7 @@
         <v>3007</v>
       </c>
       <c r="Q269" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R269"/>
       <c r="S269"/>
@@ -29182,7 +29180,7 @@
         <v>3016</v>
       </c>
       <c r="Q270" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R270"/>
       <c r="S270"/>
@@ -29204,7 +29202,7 @@
         <v>3017</v>
       </c>
       <c r="C271" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D271" t="s">
         <v>3018</v>
@@ -29246,7 +29244,7 @@
         <v>3025</v>
       </c>
       <c r="Q271" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R271"/>
       <c r="S271"/>
@@ -29402,7 +29400,7 @@
         <v>3046</v>
       </c>
       <c r="E274" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F274" t="s">
         <v>3009</v>
@@ -29460,7 +29458,7 @@
         <v>3057</v>
       </c>
       <c r="C275" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D275" t="s">
         <v>3058</v>
@@ -29502,7 +29500,7 @@
         <v>3066</v>
       </c>
       <c r="Q275" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R275"/>
       <c r="S275"/>
@@ -29524,13 +29522,13 @@
         <v>3070</v>
       </c>
       <c r="C276" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D276" t="s">
         <v>207</v>
       </c>
       <c r="E276" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F276" t="s">
         <v>3059</v>
@@ -29588,13 +29586,13 @@
         <v>3081</v>
       </c>
       <c r="C277" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D277" t="s">
         <v>3082</v>
       </c>
       <c r="E277" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F277" t="s">
         <v>3083</v>
@@ -29630,7 +29628,7 @@
         <v>3090</v>
       </c>
       <c r="Q277" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R277"/>
       <c r="S277"/>
@@ -29694,7 +29692,7 @@
         <v>3102</v>
       </c>
       <c r="Q278" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R278"/>
       <c r="S278"/>
@@ -29722,7 +29720,7 @@
         <v>3082</v>
       </c>
       <c r="E279" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F279" t="s">
         <v>3095</v>
@@ -29756,7 +29754,7 @@
         <v>3109</v>
       </c>
       <c r="Q279" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R279"/>
       <c r="S279"/>
@@ -29778,7 +29776,7 @@
         <v>3113</v>
       </c>
       <c r="C280" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D280" t="s">
         <v>2890</v>
@@ -29820,7 +29818,7 @@
         <v>3121</v>
       </c>
       <c r="Q280" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R280"/>
       <c r="S280"/>
@@ -29882,7 +29880,7 @@
         <v>3133</v>
       </c>
       <c r="Q281" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R281"/>
       <c r="S281"/>
@@ -29944,7 +29942,7 @@
         <v>3142</v>
       </c>
       <c r="Q282" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R282"/>
       <c r="S282"/>
@@ -30006,7 +30004,7 @@
         <v>3150</v>
       </c>
       <c r="Q283" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R283"/>
       <c r="S283"/>
@@ -30068,7 +30066,7 @@
         <v>3158</v>
       </c>
       <c r="Q284" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R284"/>
       <c r="S284"/>
@@ -30130,7 +30128,7 @@
         <v>3168</v>
       </c>
       <c r="Q285" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R285"/>
       <c r="S285"/>
@@ -30152,7 +30150,7 @@
         <v>3172</v>
       </c>
       <c r="C286" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D286" t="s">
         <v>3173</v>
@@ -30194,7 +30192,7 @@
         <v>3181</v>
       </c>
       <c r="Q286" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R286"/>
       <c r="S286"/>
@@ -30216,7 +30214,7 @@
         <v>3182</v>
       </c>
       <c r="C287" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D287" t="s">
         <v>3183</v>
@@ -30342,7 +30340,7 @@
         <v>3206</v>
       </c>
       <c r="C289" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D289" t="s">
         <v>3207</v>
@@ -30448,7 +30446,7 @@
         <v>3229</v>
       </c>
       <c r="Q290" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R290"/>
       <c r="S290"/>
@@ -30473,10 +30471,10 @@
         <v>113</v>
       </c>
       <c r="D291" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="E291" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F291" t="s">
         <v>3221</v>
@@ -30534,7 +30532,7 @@
         <v>3241</v>
       </c>
       <c r="C292" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D292" t="s">
         <v>536</v>
@@ -30598,13 +30596,13 @@
         <v>3252</v>
       </c>
       <c r="C293" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D293" t="s">
         <v>2701</v>
       </c>
       <c r="E293" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F293" t="s">
         <v>3221</v>
@@ -30640,7 +30638,7 @@
         <v>3259</v>
       </c>
       <c r="Q293" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R293"/>
       <c r="S293"/>
@@ -30662,7 +30660,7 @@
         <v>3263</v>
       </c>
       <c r="C294" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D294" t="s">
         <v>1261</v>
@@ -30704,7 +30702,7 @@
         <v>3270</v>
       </c>
       <c r="Q294" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R294"/>
       <c r="S294"/>
@@ -30768,7 +30766,7 @@
         <v>3281</v>
       </c>
       <c r="Q295" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R295"/>
       <c r="S295"/>
@@ -30790,7 +30788,7 @@
         <v>3282</v>
       </c>
       <c r="C296" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D296" t="s">
         <v>1836</v>
@@ -30918,19 +30916,19 @@
         <v>3299</v>
       </c>
       <c r="C298" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D298" t="s">
         <v>2865</v>
       </c>
       <c r="E298" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F298" t="s">
         <v>3300</v>
       </c>
       <c r="G298" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H298" t="s">
         <v>145</v>
@@ -30960,7 +30958,7 @@
         <v>3307</v>
       </c>
       <c r="Q298" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R298"/>
       <c r="S298"/>
@@ -31022,7 +31020,7 @@
         <v>3315</v>
       </c>
       <c r="Q299" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R299"/>
       <c r="S299"/>
@@ -31084,7 +31082,7 @@
         <v>3326</v>
       </c>
       <c r="Q300" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R300"/>
       <c r="S300"/>
@@ -31106,7 +31104,7 @@
         <v>3327</v>
       </c>
       <c r="C301" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D301" t="s">
         <v>654</v>
@@ -31272,7 +31270,7 @@
         <v>3355</v>
       </c>
       <c r="Q303" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R303"/>
       <c r="S303"/>
@@ -31356,7 +31354,7 @@
         <v>3364</v>
       </c>
       <c r="C305" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D305" t="s">
         <v>2680</v>
@@ -31398,7 +31396,7 @@
         <v>3371</v>
       </c>
       <c r="Q305" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R305"/>
       <c r="S305"/>
@@ -31482,13 +31480,13 @@
         <v>3384</v>
       </c>
       <c r="C307" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D307" t="s">
         <v>3385</v>
       </c>
       <c r="E307" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F307" t="s">
         <v>3386</v>
@@ -31524,7 +31522,7 @@
         <v>3393</v>
       </c>
       <c r="Q307" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R307"/>
       <c r="S307"/>
@@ -31586,7 +31584,7 @@
         <v>3403</v>
       </c>
       <c r="Q308" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R308"/>
       <c r="S308"/>
@@ -31714,7 +31712,7 @@
         <v>3422</v>
       </c>
       <c r="Q310" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R310"/>
       <c r="S310"/>
@@ -31736,7 +31734,7 @@
         <v>3423</v>
       </c>
       <c r="C311" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D311" t="s">
         <v>3424</v>
@@ -31800,7 +31798,7 @@
         <v>3436</v>
       </c>
       <c r="C312" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D312" t="s">
         <v>2764</v>
@@ -31812,7 +31810,7 @@
         <v>3425</v>
       </c>
       <c r="G312" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H312" t="s">
         <v>145</v>
@@ -31934,7 +31932,7 @@
         <v>3457</v>
       </c>
       <c r="E314" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F314" t="s">
         <v>3458</v>
@@ -32052,13 +32050,13 @@
         <v>3480</v>
       </c>
       <c r="C316" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D316" t="s">
         <v>1693</v>
       </c>
       <c r="E316" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F316" t="s">
         <v>3481</v>
@@ -32116,13 +32114,13 @@
         <v>3489</v>
       </c>
       <c r="C317" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D317" t="s">
         <v>2021</v>
       </c>
       <c r="E317" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F317" t="s">
         <v>3490</v>
@@ -32192,7 +32190,7 @@
         <v>3500</v>
       </c>
       <c r="G318" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H318" t="s">
         <v>115</v>
@@ -32244,13 +32242,13 @@
         <v>3511</v>
       </c>
       <c r="C319" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D319" t="s">
         <v>3512</v>
       </c>
       <c r="E319" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F319" t="s">
         <v>3513</v>
@@ -32378,7 +32376,7 @@
         <v>1757</v>
       </c>
       <c r="E321" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F321" t="s">
         <v>3537</v>
@@ -32436,7 +32434,7 @@
         <v>3545</v>
       </c>
       <c r="C322" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D322" t="s">
         <v>536</v>
@@ -32506,7 +32504,7 @@
         <v>2818</v>
       </c>
       <c r="E323" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F323" t="s">
         <v>3555</v>
@@ -32606,7 +32604,7 @@
         <v>3574</v>
       </c>
       <c r="Q324" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R324"/>
       <c r="S324"/>
@@ -32634,7 +32632,7 @@
         <v>2701</v>
       </c>
       <c r="E325" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F325" t="s">
         <v>3576</v>
@@ -32696,7 +32694,7 @@
         <v>1693</v>
       </c>
       <c r="E326" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F326" t="s">
         <v>3584</v>
@@ -32730,7 +32728,7 @@
         <v>3590</v>
       </c>
       <c r="Q326" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R326"/>
       <c r="S326"/>
@@ -32752,7 +32750,7 @@
         <v>3591</v>
       </c>
       <c r="C327" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D327" t="s">
         <v>3499</v>
@@ -32764,7 +32762,7 @@
         <v>3592</v>
       </c>
       <c r="G327" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H327" t="s">
         <v>115</v>
@@ -32816,7 +32814,7 @@
         <v>3603</v>
       </c>
       <c r="C328" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D328" t="s">
         <v>3604</v>
@@ -32858,7 +32856,7 @@
         <v>3612</v>
       </c>
       <c r="Q328" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R328"/>
       <c r="S328"/>
@@ -32922,7 +32920,7 @@
         <v>3625</v>
       </c>
       <c r="Q329" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R329"/>
       <c r="S329"/>
@@ -32944,13 +32942,13 @@
         <v>3626</v>
       </c>
       <c r="C330" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D330" t="s">
         <v>3627</v>
       </c>
       <c r="E330" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F330" t="s">
         <v>3628</v>
@@ -32986,7 +32984,7 @@
         <v>3635</v>
       </c>
       <c r="Q330" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R330"/>
       <c r="S330"/>
@@ -33050,7 +33048,7 @@
         <v>3644</v>
       </c>
       <c r="Q331" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R331"/>
       <c r="S331"/>
@@ -33072,7 +33070,7 @@
         <v>3645</v>
       </c>
       <c r="C332" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D332" t="s">
         <v>3646</v>
@@ -33136,19 +33134,19 @@
         <v>3657</v>
       </c>
       <c r="C333" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D333" t="s">
         <v>2865</v>
       </c>
       <c r="E333" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F333" t="s">
         <v>3637</v>
       </c>
       <c r="G333" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H333" t="s">
         <v>247</v>
@@ -33200,7 +33198,7 @@
         <v>3668</v>
       </c>
       <c r="C334" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D334" t="s">
         <v>2722</v>
@@ -33242,7 +33240,7 @@
         <v>3675</v>
       </c>
       <c r="Q334" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R334"/>
       <c r="S334"/>
@@ -33264,13 +33262,13 @@
         <v>3679</v>
       </c>
       <c r="C335" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D335" t="s">
         <v>1540</v>
       </c>
       <c r="E335" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F335" t="s">
         <v>3680</v>
@@ -33370,7 +33368,7 @@
         <v>3697</v>
       </c>
       <c r="Q336" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="R336"/>
       <c r="S336"/>
@@ -33392,7 +33390,7 @@
         <v>3698</v>
       </c>
       <c r="C337" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D337" t="s">
         <v>536</v>
@@ -33434,7 +33432,7 @@
         <v>3706</v>
       </c>
       <c r="Q337" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R337"/>
       <c r="S337"/>
@@ -33456,7 +33454,7 @@
         <v>3707</v>
       </c>
       <c r="C338" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D338" t="s">
         <v>1811</v>
@@ -33526,7 +33524,7 @@
         <v>3082</v>
       </c>
       <c r="E339" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F339" t="s">
         <v>3717</v>
@@ -33584,7 +33582,7 @@
         <v>3728</v>
       </c>
       <c r="C340" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D340" t="s">
         <v>2033</v>
@@ -33626,7 +33624,7 @@
         <v>3735</v>
       </c>
       <c r="Q340" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="R340"/>
       <c r="S340"/>
@@ -33648,7 +33646,7 @@
         <v>3736</v>
       </c>
       <c r="C341" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D341" t="s">
         <v>536</v>

</xml_diff>

<commit_message>
Update parliament data - 2026-06-28
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -1016,10 +1016,10 @@
     <t xml:space="preserve">2025-12-17</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&amp;gt; Das Ruder wieder übernehmen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&amp;gt;  Il est temps de reprendre les choses en main</t>
+    <t xml:space="preserve">xml:space="preserve"&gt; Das Ruder wieder übernehmen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;  Il est temps de reprendre les choses en main</t>
   </si>
   <si>
     <t xml:space="preserve">È tempo di prendere in mano la situazione</t>
@@ -1509,10 +1509,10 @@
     <t xml:space="preserve">25.3893</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&amp;gt; Transparenz und Rechtfertigung der finanziellen Reserven der Suva und Prüfung durch die Eidgenössische Finanzkontrolle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&amp;gt; Transparence et justification des réserves financières de la Suva et contrôle du CDF</t>
+    <t xml:space="preserve">xml:space="preserve"&gt; Transparenz und Rechtfertigung der finanziellen Reserven der Suva und Prüfung durch die Eidgenössische Finanzkontrolle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt; Transparence et justification des réserves financières de la Suva et contrôle du CDF</t>
   </si>
   <si>
     <t xml:space="preserve">Trasparenza e giustificazione delle riserve finanziarie della Suva e controllo del CDF</t>
@@ -1848,13 +1848,13 @@
     <t xml:space="preserve">Schmezer Ueli</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;CO2-Verordnung. Erleichterungsmassnahmen für die Autobranche? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Ordonnance sur le CO2. Des mesures d'allègement pour la branche automobile ? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Ordinanza sul CO2. Misure di agevolazione per il settore automobilistico? </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;CO2-Verordnung. Erleichterungsmassnahmen für die Autobranche? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Ordonnance sur le CO2. Des mesures d'allègement pour la branche automobile ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Ordinanza sul CO2. Misure di agevolazione per il settore automobilistico? </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;La révision, ou plus précisément l’adaptation de l’ordonnance sur le CO2 faisant suite à la révision de la loi sur le CO2 (en vigueur depuis le 1.1.2025), revêt une grande importance pour la réalisation des objectifs légaux en matière d'émissions. Cela concerne en particulier les dispositions d'exécution pour les voitures de tourisme.&amp;amp;amp;nbsp;&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;Le 17 mars 2025, le Conseil fédéral a laissé entendre pendant l’heure des questions qu'il « adopterait l'ordonnance lors d'une prochaine séance ». Il a répondu de façon évasive aux questions sur cette ordonnance.&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;La présente interpellation s’intéresse aux mesures d'allègement des sanctions pécuniaires qui pourraient éventuellement être (une nouvelle fois) accordées à la branche automobile lorsque celle-ci ne parvient pas à atteindre les valeurs cibles.&amp;amp;amp;nbsp;&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;Concrètement, l’ordonnance sur le CO2 soulève les questions suivantes.&amp;amp;amp;nbsp;&amp;amp;lt;br&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;ol&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;La procédure de consultation s’est achevée le 17 octobre 2024. Pourquoi cette ordonnance dont nous avons urgemment besoin n'est-elle pas entrée en vigueur en mars 2025&amp;amp;amp;nbsp;? Quels sont les facteurs qui ont conduit à ce retard.&amp;amp;amp;nbsp;&amp;amp;lt;br&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Le projet envoyé en consultation ne prévoyait pas d'alléger les sanctions. Sur les 202 prises de position annoncées par le Conseil fédéral, combien demandaient, dans le délai imparti par la procédure, des allégements en cas de non-respect des objectifs ? Quels étaient leurs principaux arguments ?&amp;amp;amp;nbsp;&amp;amp;lt;br&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Le Contrôle fédéral des finances (CDF) a évalué l'efficacité des sanctions en matière de CO2 pour les voitures de tourisme neuves : il est clair pour lui qu'il faut renoncer à des mesures d'allégement si les objectifs ne sont pas atteints.&amp;amp;amp;nbsp;&amp;amp;lt;br&amp;amp;gt;Le Conseil fédéral partage-t-il l'appréciation du CDF ? Si ce n'est pas le cas, quels sont ses arguments ?&amp;amp;lt;br&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Par le passé (notamment en 2015 et en 2020), des dispositions prévoyant des allégements (supercrédits, phase d’introduction) ont été introduites pour réduire les montants des sanctions en cas de dépassement des objectifs d'émission. Quel est le montant cumulé des dépassements d'objectifs non sanctionnés depuis 2010 en Suisse&amp;amp;amp;nbsp;?&amp;amp;amp;nbsp;&amp;amp;lt;br&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Si le Conseil fédéral introduit des mesures d'allégement dans l'ordonnance : combien de millions de francs d’exonérations cela représentera-t-il pour la branche&amp;amp;amp;nbsp;?&amp;amp;lt;br&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Si le Conseil fédéral introduit des mesures d'allégement dans l'ordonnance : comment sera-t-il possible, d’après lui, d’atteindre les valeurs cibles prévues par la loi&amp;amp;amp;nbsp;?&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;/ol&amp;amp;gt;</t>
@@ -2163,10 +2163,10 @@
     <t xml:space="preserve">2025-03-11</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Nimmt der Bundesrat die Finanzkontrolle ernst? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Le Conseil fédéral prend-il au sérieux le Contrôle fédéral des finances ? </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Nimmt der Bundesrat die Finanzkontrolle ernst? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Le Conseil fédéral prend-il au sérieux le Contrôle fédéral des finances ? </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;L'élaboration de l'ordonnance sur le CO2 revêt une grande importance pour la réalisation des objectifs légaux en matière d'émissions, en particulier les dispositions d'exécution pour les voitures de tourisme.&amp;amp;lt;br&amp;amp;gt;Le Contrôle fédéral des finances a évalué l'efficacité des sanctions en matière de CO2 pour les voitures de tourisme neuves&amp;amp;amp;nbsp;: il est clair pour lui qu'il faut renoncer à des mesures d'allègement si les objectifs ne sont pas atteints.&amp;amp;lt;br&amp;amp;gt;Le Conseil fédéral partage-t-il l'avis du Contrôle fédéral des finances&amp;amp;amp;nbsp;? Dans la négative, pour quelles raisons&amp;amp;amp;nbsp;?&amp;amp;lt;/p&amp;amp;gt;</t>
@@ -2262,10 +2262,10 @@
     <t xml:space="preserve">25.7129</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Ist der Kaufpreis für die F-35 fix? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Le prix d’achat des F-35, est-il fixe ? </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Ist der Kaufpreis für die F-35 fix? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Le prix d’achat des F-35, est-il fixe ? </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;Selon les informations régulièrement transmises par le DDPS, les Etats-Unis se sont engagés à fournir les 36 F-35 acquis par la Suisse à un prix d’achat fixe. Mais selon un avis du Contrôle fédéral des finances émis le 8 juillet 2022, il n’existe aucune garantie juridique à ce sujet.&amp;amp;lt;br&amp;amp;gt;A notre connaissance, cette dernière information n’a jamais été démentie par le Conseil fédéral.&amp;amp;lt;br&amp;amp;gt;Le Conseil fédéral la confirme-t-il ?&amp;amp;lt;/p&amp;amp;gt;</t>
@@ -2397,13 +2397,13 @@
     <t xml:space="preserve">2025-01-21</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Schweizer Depotbank für die Ausgleichfonds von AHV, IV und EO </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Schweizer Depotbank für die Ausgleichfonds von AHV, IV und EO </t>
   </si>
   <si>
     <t xml:space="preserve">Banque dépositaire pour les fonds de compensation AVS/AI/APG</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Banca depositaria svizzera per i fondi di compensazione AVS, AI e IPG </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Banca depositaria svizzera per i fondi di compensazione AVS, AI e IPG </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;Les fonds de compensation AVS/AI/APG sont responsables de la gestion des liquidités et de la fortune de ces trois assurances. En décembre&amp;amp;amp;nbsp;2023, le conseil d’administration de Compenswiss, l’autorité compétente, a décidé de confier le mandat de banque dépositaire, qui était alors assumé par UBS, à un établissement bancaire américain, la State Street Bank International GmbH. Le transfert à la nouvelle banque dépositaire a eu lieu fin juillet&amp;amp;amp;nbsp;2024.&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;Le Conseil fédéral est chargé d’encourager Compenswiss à résilier le mandat confié à la State Street Bank International GmbH pour le remettre à une banque suisse. Si, pour des raisons juridiques, cela n’est pas possible, le Conseil fédéral est chargé de créer les conditions légales nécessaires.&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;Une minorité (Bertschy, Grossen Jürg, Roth David, Ryser, Walti Beat, Wermuth, Widmer Céline) propose de rejeter la motion.&amp;amp;lt;/p&amp;amp;gt;</t>
@@ -2499,10 +2499,10 @@
     <t xml:space="preserve">2024-12-11</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;ETH-Top vs. ETH-Baumanagement-Flop </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;EPFZ. Un top et un flop </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;ETH-Top vs. ETH-Baumanagement-Flop </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;EPFZ. Un top et un flop </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;Top&amp;amp;amp;nbsp;: 7e place dans le classement mondial des universités 2025. Flop&amp;amp;amp;nbsp;: l’EPFZ comme maître d’ouvrage. 2019&amp;amp;amp;nbsp;: rapport du CDF à propos du projet BSS (Bâle)&amp;amp;amp;nbsp;: «&amp;amp;amp;nbsp;la direction du projet BSS n’a pas mis en œuvre de processus valables pour la gestion du changement&amp;amp;amp;nbsp;»&amp;amp;amp;nbsp;; «&amp;amp;amp;nbsp;il n’existe pas d’instruments continus pour le pilotage financier de l’ensemble du projet ». 2023-2024&amp;amp;amp;nbsp;: projet GLC (Zurich)&amp;amp;amp;nbsp;: une centaine de PME et d’entreprises générales attendent encore le versement de plusieurs millions de francs. L’EPFZ refuse de donner suite aux demandes d’entretien des entreprises générales en vue de résoudre le problème.&amp;amp;lt;br&amp;amp;gt;Que fait le Conseil fédéral pour protéger les entreprises concernées et la réputation de l’EPFZ&amp;amp;amp;nbsp;?&amp;amp;lt;/p&amp;amp;gt;</t>
@@ -3408,10 +3408,10 @@
     <t xml:space="preserve">2024-02-26</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Unterstellung von Organisationen ausserhalb der Bundesverwaltung unter die Aufsicht durch die Eidgenössische Finanzkontrolle. Wann wird der Bundesrat seinen Bericht veröffentlichen? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Assujettissement des organisations externes à l’administration au Contrôle fédéral des finances. Quand le Conseil fédéral publiera-t-il son rapport ? </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Unterstellung von Organisationen ausserhalb der Bundesverwaltung unter die Aufsicht durch die Eidgenössische Finanzkontrolle. Wann wird der Bundesrat seinen Bericht veröffentlichen? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Assujettissement des organisations externes à l’administration au Contrôle fédéral des finances. Quand le Conseil fédéral publiera-t-il son rapport ? </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;Le postulat 15.4112 intitulé «&amp;amp;amp;nbsp;Examen des critères selon lesquels les organisations externes à l’administration doivent être soumises à la surveillance du Contrôle fédéral des finances&amp;amp;amp;nbsp;» a été accepté par le Conseil national le 18 mars 2016. En réponse à la question 19.5385, le Conseil fédéral a indiqué que le rapport demandé par le postulat serait publié à la fin de l’année 2019. Pour l’heure, le rapport n’a pas encore été publié.&amp;amp;lt;br&amp;amp;gt;Quand le sera-t-il&amp;amp;amp;nbsp;?&amp;amp;amp;nbsp;&amp;amp;lt;/p&amp;amp;gt;</t>
@@ -3594,7 +3594,7 @@
     <t xml:space="preserve">Fonds pour la démocratie et l'état de droit en commémoration de 1848</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&amp;gt; Fondo per la democrazia e lo Stato di diritto in commemorazione del 1848</t>
+    <t xml:space="preserve">xml:space="preserve"&gt; Fondo per la democrazia e lo Stato di diritto in commemorazione del 1848</t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;Le Conseil fédéral est invité à élaborer les bases légales pour le financement d’un fonds pour la démocratie et l’État de droit. Ce fonds doit, d’une part, soutenir des activités pouvant renforcer la compréhension et l’engagement pour les institutions politiques de l’État fédéral suisse, en particulier chez les jeunes. D’autre part, afin de renforcer la cohésion de la Suisse, le fonds doit encourager la connaissance et la pratique des langues nationales.&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;&amp;amp;amp;nbsp;&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;Le fonds doit être géré par un comité indépendant du Parlement et de l’administration, composé de cinq à neuf personnes au maximum, nommées par le Conseil fédéral pour une durée de quatre ans et rééligibles deux fois au maximum. Les comptes annuels doivent être soumis au Contrôle fédéral des finances pour révision.&amp;amp;lt;/p&amp;amp;gt;</t>
@@ -3630,7 +3630,7 @@
     <t xml:space="preserve">Une manifestation en faveur du pouvoir d'achat doit-elle être considérée comme une manifestation électorale?</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Una manifestazione a favore del potere d'acquisto è una manifestazione elettorale o no? </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Una manifestazione a favore del potere d'acquisto è una manifestazione elettorale o no? </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;Dans le « Tagesanzeiger » du 22 septembre 2023, le directeur du Contrôle fédéral des finances, Pascal Stirnimann, a affirmé, à propos d’une manifestation en faveur du pouvoir d’achat qui a été organisée par l’Union syndicale suisse (USS) et à laquelle participaient des parlementaires fédéraux socialistes et verts, que si, lors d’une grande manifestation, dix candidats d’un même parti scandaient leurs slogans électoraux, mais que les organisateurs de la manifestation affirmaient néanmoins qu’il ne s’agissait pas d’une campagne électorale, le CDF allait examiner la chose de près.&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;p&amp;amp;gt;Dans ce contexte, je prie le Conseil fédéral de répondre aux questions suivantes&amp;amp;amp;nbsp;:&amp;amp;amp;nbsp;&amp;amp;lt;/p&amp;amp;gt;&amp;amp;lt;ol&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;A-t-on, après la manifestation sur le pouvoir d’achat organisée par les syndicats, ouvert une enquête pour déterminer si la loi sur le financement de la vie politique avait été violée&amp;amp;amp;nbsp;?&amp;amp;lt;br&amp;amp;gt;a. Dans l’affirmative, pourquoi&amp;amp;amp;nbsp;?&amp;amp;lt;br&amp;amp;gt;b. Dans la négative, pourquoi&amp;amp;amp;nbsp;?&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Dans le cas où une enquête a été ouverte, quand disposera-t-on, selon le Conseil fédéral, des premiers résultats&amp;amp;amp;nbsp;?&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Selon lui, une manifestation disposant d’un budget de 150&amp;amp;amp;nbsp;000&amp;amp;amp;nbsp;francs (comme ce fut le cas pour la manifestation en faveur du pouvoir d’achat) doit-elle faire l’objet d’une déclaration conformément à la loi sur le financement de la vie politique&amp;amp;amp;nbsp;?&amp;amp;amp;nbsp;&amp;amp;lt;br&amp;amp;gt;a. Dans l’affirmative, pourquoi&amp;amp;amp;nbsp;?&amp;amp;lt;br&amp;amp;gt;b. Dans la négative, pourquoi&amp;amp;amp;nbsp;?&amp;amp;amp;nbsp;&amp;amp;amp;nbsp;&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Le Conseil fédéral approuve-t-il l’affirmation de Pascal Stirnimann selon laquelle toute personne qui dépense, en vue d’influer sur une élection, des montants dépassant les plafonds fixés par la loi est tenue de les déclarer&amp;amp;amp;nbsp;?&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Où se situe, pour le Conseil fédéral, la limite entre une manifestation ne visant pas à influer sur une élection et une manifestation visant une telle fin&amp;amp;amp;nbsp;?&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Que pense-t-il de l’argument avancé par le porte-parole de l’USS selon lequel ladite manifestation portait sur les négociations salariales, qu’elle ne constituait pas une manifestation électorale au sens de la loi et qu’elle ne devait, par conséquent, pas faire l’objet d’une déclaration&amp;amp;amp;nbsp;?&amp;amp;amp;nbsp;&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;li&amp;amp;gt;Est-il d’avis que toutes les manifestations susceptibles d’être considérées comme des manifestations électorales en raison de leur rayonnement ou du sujet sur lequel elles portent sont soumises à la loi sur le financement de la vie politique&amp;amp;amp;nbsp;?&amp;amp;lt;/li&amp;amp;gt;&amp;amp;lt;/ol&amp;amp;gt;</t>
@@ -4254,7 +4254,7 @@
     <t xml:space="preserve">Die Schweizerische Radio- und Fernsehgesellschaft der Eidgenössischen Finanzkontrolle unterstellen</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Soumettre la Société suisse de radiodiffusion et télévision au Contrôle fédéral des finances </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Soumettre la Société suisse de radiodiffusion et télévision au Contrôle fédéral des finances </t>
   </si>
   <si>
     <t xml:space="preserve">Società svizzera di radiotelevisione da sottoporre al Controllo federale delle finanze</t>
@@ -7572,10 +7572,10 @@
     <t xml:space="preserve">25.8273</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Kostendeckende Erträge aus dem Artenschutz? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Des revenus couvrant les coûts liés à la protection des espèces ? </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Kostendeckende Erträge aus dem Artenschutz? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Des revenus couvrant les coûts liés à la protection des espèces ? </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;Chaque année, la Suisse délivre environ 100&amp;amp;amp;nbsp;000 autorisations pour le commerce d'espèces végétales et animales menacées et effectue quelque 20&amp;amp;amp;nbsp;000 contrôles à l'importation. Elle perçoit à cet effet des émoluments d'environ 4&amp;amp;amp;nbsp;millions de francs. Selon le CDF, ces émoluments ne couvriraient pas les coûts et constitueraient donc une subvention dommageable à la biodiversité.&amp;amp;lt;br&amp;amp;gt;Compte tenu des débats en cours concernant le budget,&amp;amp;lt;br&amp;amp;gt;le Conseil fédéral est-il prêt à introduire des émoluments couvrant les coûts dans ce domaine&amp;amp;amp;nbsp;?&amp;amp;lt;br&amp;amp;gt;Si oui, quand&amp;amp;amp;nbsp;?&amp;amp;lt;br&amp;amp;gt;Si non, pourquoi&amp;amp;amp;nbsp;?&amp;amp;lt;/p&amp;amp;gt;</t>
@@ -7740,10 +7740,10 @@
     <t xml:space="preserve">25.4225</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Giftiger Rasen. Warum sind toxische PFAS-Pestizide ausgerechnet zur Anwendung auf Spiel- und Sportplätzen oder in Wohnquartieren zugelassen? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Gazon toxique. Pourquoi les pesticides PFAS sont-ils autorisés sur les terrains de jeux et de sport ainsi que dans les quartiers résidentiels ? </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Giftiger Rasen. Warum sind toxische PFAS-Pestizide ausgerechnet zur Anwendung auf Spiel- und Sportplätzen oder in Wohnquartieren zugelassen? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Gazon toxique. Pourquoi les pesticides PFAS sont-ils autorisés sur les terrains de jeux et de sport ainsi que dans les quartiers résidentiels ? </t>
   </si>
   <si>
     <t xml:space="preserve">Superfici erbose inquinate. Perché i pesticidi tossici contenenti PFAS sono omologati per l'uso sui campi sportivi e da gioco e nei quartieri residenziali?</t>
@@ -7926,10 +7926,10 @@
     <t xml:space="preserve">25.789</t>
   </si>
   <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Rolle des Bundes bei der Sanierung der Deponie Gamsenried </t>
-  </si>
-  <si>
-    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&amp;gt;Rôle de la Confédération dans l’assainissement de la décharge de Gamsenried </t>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Rolle des Bundes bei der Sanierung der Deponie Gamsenried </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;xml:space="preserve"&gt;Rôle de la Confédération dans l’assainissement de la décharge de Gamsenried </t>
   </si>
   <si>
     <t xml:space="preserve">&amp;amp;lt;p&amp;amp;gt;Concernant le suivi de l’assainissement de cette décharge, le Contrôle fédéral des finances (CDF) souligne «&amp;amp;amp;nbsp;l’absence d’une vision d’ensemble des risques et d’un suivi coordonné des différentes entités fédérales&amp;amp;amp;nbsp;».&amp;amp;lt;br&amp;amp;gt;- Comment le Conseil fédéral réagit-il aux critiques du CDF?&amp;amp;lt;br&amp;amp;gt;- Entend-il réaliser une analyse globale des risques, en tenant compte des interfaces avec l'A9 et la correction du Rhône puis, sur cette base, établir un concept de surveillance avec des responsabilités clairement définies?&amp;amp;lt;/p&amp;amp;gt;</t>
@@ -11430,10 +11430,10 @@
     <t xml:space="preserve">Sottoporre la SUVA alla vigilanza finanziaria del Controllo federale delle finanze</t>
   </si>
   <si>
-    <t xml:space="preserve">&amp;lt;p&amp;gt;Le Conseil fédéral est chargé de proposer aux Chambres fédérales d'abroger l'article 1, alinéa , lettera , de la loi sur le Contrôle des finances (LCF ; RS 614.0) lorsqu'elles procéderont à la prochaine révision de la loi en question.&amp;lt;/p&amp;gt;&amp;lt;p&amp;gt;Une minorité (Gasche, Gilli, Gmür, Gössi, Gschwind, Kiener Nellen, Müller Leo, Schneeberger, Siegenthaler, Vischer Daniel) propose le rejet de la motion.&amp;lt;/p&amp;gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&amp;lt;p&amp;gt;Der Bundesrat wird beauftragt, der Bundesversammlung im Rahmen der nächsten Revision des Finanzkontrollgesetzes (FKG; SR 614.0) die ersatzlose Streichung von Artikel 19 Absatz 1 Buchstabe b vorzulegen.&amp;lt;/p&amp;gt;&amp;lt;p&amp;gt;Eine Minderheit (Gasche, Gilli, Gmür, Gössi, Gschwind, Kiener Nellen, Müller Leo, Schneeberger, Siegenthaler, Vischer Daniel) beantragt die Ablehnung der Motion.&amp;lt;/p&amp;gt;</t>
+    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de proposer aux Chambres fédérales d'abroger l'article 1, alinéa , lettera , de la loi sur le Contrôle des finances (LCF ; RS 614.0) lorsqu'elles procéderont à la prochaine révision de la loi en question.&lt;/p&gt;&lt;p&gt;Une minorité (Gasche, Gilli, Gmür, Gössi, Gschwind, Kiener Nellen, Müller Leo, Schneeberger, Siegenthaler, Vischer Daniel) propose le rejet de la motion.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, der Bundesversammlung im Rahmen der nächsten Revision des Finanzkontrollgesetzes (FKG; SR 614.0) die ersatzlose Streichung von Artikel 19 Absatz 1 Buchstabe b vorzulegen.&lt;/p&gt;&lt;p&gt;Eine Minderheit (Gasche, Gilli, Gmür, Gössi, Gschwind, Kiener Nellen, Müller Leo, Schneeberger, Siegenthaler, Vischer Daniel) beantragt die Ablehnung der Motion.&lt;/p&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20153828</t>
@@ -11472,10 +11472,10 @@
     <t xml:space="preserve">Bloccare l'effettivo del personale della Confederazione al livello del 2015</t>
   </si>
   <si>
-    <t xml:space="preserve">&amp;lt;p&amp;gt;Le Conseil fédéral est chargé de prendre des mesures afin que les effectifs de la Confédération ne dépassent pas le nombre fixé dans le budget 2015 (à savoir 35 000 équivalents plein temps).&amp;lt;/p&amp;gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&amp;lt;p&amp;gt;Der Bundesrat wird beauftragt, Massnahmen zu ergreifen mit dem Ziel, dass der Bundespersonalbestand den Stand gemäss Voranschlag 2015 (35 000 FTE) nicht überschreitet.&amp;lt;/p&amp;gt;</t>
+    <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé de prendre des mesures afin que les effectifs de la Confédération ne dépassent pas le nombre fixé dans le budget 2015 (à savoir 35 000 équivalents plein temps).&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, Massnahmen zu ergreifen mit dem Ziel, dass der Bundespersonalbestand den Stand gemäss Voranschlag 2015 (35 000 FTE) nicht überschreitet.&lt;/p&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.parlament.ch/de/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20153494</t>

</xml_diff>

<commit_message>
Update parliament data - 2026-07-06
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -257,10 +257,10 @@
     <t xml:space="preserve">Titel folgt</t>
   </si>
   <si>
-    <t xml:space="preserve">Réintroduction de l’obligation de visas pour les Géorgiens </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reintrodurre l’obbligo del visto per i Georgiani</t>
+    <t xml:space="preserve">Réintroduction de l'obligation de visas pour les Géorgiens </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reintrodurre l'obbligo del visto per i Georgiani</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Le Conseil fédéral est chargé d’intervenir auprès de l’Union européenne afin de demander la réintroduction de l’obligation de visas pour les ressortissants géorgiens. Cette mesure vise à enrayer le tourisme médical qui n’a pas tari.&lt;/p&gt;</t>

</xml_diff>

<commit_message>
Update parliament data - 2026-07-10
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -104,7 +104,7 @@
     <t xml:space="preserve">UVEK</t>
   </si>
   <si>
-    <t xml:space="preserve">Gotthard-Eisenbahnachse: Plant der Bundesrat, die bei der Ausarbeitung der Botschaft 2027 aufgetretenen Mängel zu beheben?</t>
+    <t xml:space="preserve">Gotthard-Eisenbahnachse. Plant der Bundesrat, die bei der Ausarbeitung der Botschaft 2027 aufgetretenen Mängel zu beheben?</t>
   </si>
   <si>
     <t xml:space="preserve">Axe ferroviaire du Saint-Gothard. Le Conseil fédéral a-t-il l'intention de remédier aux lacunes constatées lors de la préparation du message 2027 ?</t>
@@ -248,7 +248,7 @@
     <t xml:space="preserve">Titre suit</t>
   </si>
   <si>
-    <t xml:space="preserve">Attuazione coerente dell’Agenda 2030 nelle politiche settoriali</t>
+    <t xml:space="preserve">Attuazione coerente dell'Agenda 2030 nelle politiche settoriali</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Der Bundesrat wird beauftragt, Massnahmen zu ergreifen, um eine umfassende, kohärente und wirkungsvolle Umsetzung der Agenda 2030 in den Sektoralpolitiken sicherzustellen:&amp;nbsp;&lt;/p&gt;&lt;ol style="list-style-type:decimal;"&gt;&lt;li&gt;Auf Basis des Länderberichts (Voluntary National Review) 2026 ist eine gezielte Analyse der notwendigen Massnahmen vorzunehmen, um die festgestellten Lücken zu schliessen.&amp;nbsp;&lt;/li&gt;&lt;li&gt;Der Bundesrat muss sicherstellen, dass das Direktionskomitee Agenda 2030 seine koordinierende und steuernde Rolle wahrnimmt und die Agenda 2030 kohärent in die Sektoralpolitiken übersetzt.&amp;nbsp;&lt;/li&gt;&lt;li&gt;Der Bundesrat muss dem Parlament in regelmässigen Abständen über die zusätzlichen Massnahmen berichten.&amp;nbsp;&lt;/li&gt;&lt;/ol&gt;</t>

</xml_diff>

<commit_message>
Update parliament data - 2026-08-13
</commit_message>
<xml_diff>
--- a/Objets_parlementaires_CDF_EFK.xlsx
+++ b/Objets_parlementaires_CDF_EFK.xlsx
@@ -12025,9 +12025,7 @@
       <c r="R2" t="s">
         <v>39</v>
       </c>
-      <c r="S2" t="s">
-        <v>39</v>
-      </c>
+      <c r="S2"/>
       <c r="T2" t="s">
         <v>40</v>
       </c>

</xml_diff>